<commit_message>
Improve the rendering of multiple recommendations
</commit_message>
<xml_diff>
--- a/data/league-new-player-data-template-populated.xlsx
+++ b/data/league-new-player-data-template-populated.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30524"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="149" documentId="11_91E030B3067DB12A649EB0356813936805D8A028" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ED6D6D84-6D03-4542-BF3B-1468C39B97CC}"/>
+  <xr:revisionPtr revIDLastSave="531" documentId="11_91E030B3067DB12A649EB0356813936805D8A028" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E744ABE-3E4F-40CD-9902-CCD5DBAEF82F}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" firstSheet="5" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -16,6 +16,7 @@
     <sheet name="Builds" sheetId="6" r:id="rId6"/>
     <sheet name="BuildItems" sheetId="7" r:id="rId7"/>
     <sheet name="Lists" sheetId="8" state="hidden" r:id="rId8"/>
+    <sheet name="Runes" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -171,7 +172,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000002000000}">
+    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000002000000}">
       <text>
         <r>
           <rPr>
@@ -214,7 +215,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="348">
   <si>
     <t>Topic</t>
   </si>
@@ -465,6 +466,12 @@
     <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/Darius.png</t>
   </si>
   <si>
+    <t>Malphite.png</t>
+  </si>
+  <si>
+    <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/Malphite.png</t>
+  </si>
+  <si>
     <t>warwick</t>
   </si>
   <si>
@@ -495,7 +502,7 @@
     <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/Amumu.png</t>
   </si>
   <si>
-    <t>master yi</t>
+    <t>master-yi</t>
   </si>
   <si>
     <t>Master Yi</t>
@@ -510,6 +517,90 @@
     <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/MasterYi.png</t>
   </si>
   <si>
+    <t>annie</t>
+  </si>
+  <si>
+    <t>Annie</t>
+  </si>
+  <si>
+    <t>Annie has simple abilities, reliable damage, and a powerful stun</t>
+  </si>
+  <si>
+    <t>Annie.png</t>
+  </si>
+  <si>
+    <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/Annie.png</t>
+  </si>
+  <si>
+    <t>Lux has strong abilities,which include a stun and allow her a high damage output from a safe distance</t>
+  </si>
+  <si>
+    <t>Lux.png</t>
+  </si>
+  <si>
+    <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/Lux.png</t>
+  </si>
+  <si>
+    <t>malzahar</t>
+  </si>
+  <si>
+    <t>Malzahar</t>
+  </si>
+  <si>
+    <t>Malzahar has straightforward gameplay, easy wave clearing and a targeted ultimate ability that can lock down enemy champions</t>
+  </si>
+  <si>
+    <t>Malzahar.png</t>
+  </si>
+  <si>
+    <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/Malzahar</t>
+  </si>
+  <si>
+    <t>ashe</t>
+  </si>
+  <si>
+    <t>Ashe</t>
+  </si>
+  <si>
+    <t>Ashe has straightforward abilities, long attack range, and useful crowd control</t>
+  </si>
+  <si>
+    <t>Ashe.png</t>
+  </si>
+  <si>
+    <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/Ashe.png</t>
+  </si>
+  <si>
+    <t>miss-fortune</t>
+  </si>
+  <si>
+    <t>Miss Fortune</t>
+  </si>
+  <si>
+    <t>Miss Fortune has simple abilities, strong lane presence, and a powerful ultimate that is easy to use in team fights</t>
+  </si>
+  <si>
+    <t>MissFortune.png</t>
+  </si>
+  <si>
+    <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/MissFortune.png</t>
+  </si>
+  <si>
+    <t>caitlyn</t>
+  </si>
+  <si>
+    <t>Caitlyn</t>
+  </si>
+  <si>
+    <t>Caitlyn's long attack range makes farming and bullying opponents safer</t>
+  </si>
+  <si>
+    <t>Caitlyn.png</t>
+  </si>
+  <si>
+    <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/Caitlyn.png</t>
+  </si>
+  <si>
     <t>DisplayName</t>
   </si>
   <si>
@@ -594,6 +685,12 @@
     <t>Why</t>
   </si>
   <si>
+    <t>KeystoneRuneId</t>
+  </si>
+  <si>
+    <t>RuneReason</t>
+  </si>
+  <si>
     <t>ReviewedBy</t>
   </si>
   <si>
@@ -621,6 +718,9 @@
     <t>REC003</t>
   </si>
   <si>
+    <t>Easy-Meduim</t>
+  </si>
+  <si>
     <t>Tank</t>
   </si>
   <si>
@@ -630,15 +730,114 @@
     <t>REC004</t>
   </si>
   <si>
-    <t>Easy-Meduim</t>
-  </si>
-  <si>
     <t>Enhancing</t>
   </si>
   <si>
     <t>Strong shielding and relatively easy to understand</t>
   </si>
   <si>
+    <t>conqueror</t>
+  </si>
+  <si>
+    <t>REC005</t>
+  </si>
+  <si>
+    <t>Fighter/Tank</t>
+  </si>
+  <si>
+    <t>Powerful fighter with a simple but effective kit</t>
+  </si>
+  <si>
+    <t>REC006</t>
+  </si>
+  <si>
+    <t>Simple abilitie kit, strong durability, and no resource managment</t>
+  </si>
+  <si>
+    <t>REC007</t>
+  </si>
+  <si>
+    <t>excellent survivability, and straightforward abilities</t>
+  </si>
+  <si>
+    <t>REC008</t>
+  </si>
+  <si>
+    <t>Fighter</t>
+  </si>
+  <si>
+    <t>Much sustain through healing, and a simple jungle clear</t>
+  </si>
+  <si>
+    <t>REC009</t>
+  </si>
+  <si>
+    <t>Simple abilities, strong crowd control, and his tankiness is forgiving</t>
+  </si>
+  <si>
+    <t>REC010</t>
+  </si>
+  <si>
+    <t>Straightforward kit which is focused on dealing damage and farming</t>
+  </si>
+  <si>
+    <t>REC011</t>
+  </si>
+  <si>
+    <t>Mage</t>
+  </si>
+  <si>
+    <t>Simple abilities, reliable damage, and a powerful stun</t>
+  </si>
+  <si>
+    <t>REC012</t>
+  </si>
+  <si>
+    <t>Long range abilities that allow to safely damage enemies</t>
+  </si>
+  <si>
+    <t>REC013</t>
+  </si>
+  <si>
+    <t>Easy wave clearing and a targeted lock down ultimate</t>
+  </si>
+  <si>
+    <t>REC014</t>
+  </si>
+  <si>
+    <t>Ranged Fighter</t>
+  </si>
+  <si>
+    <t>Straightforward abilities, long attack range, and crowd control</t>
+  </si>
+  <si>
+    <t>REC015</t>
+  </si>
+  <si>
+    <t>Simple abilities,strong lane presence, and a powerful ultimate</t>
+  </si>
+  <si>
+    <t>REC016</t>
+  </si>
+  <si>
+    <t>Long attack range, easy farming, good lane control</t>
+  </si>
+  <si>
+    <t>REC017</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>REC018</t>
+  </si>
+  <si>
+    <t>Much sustain through healing, and an easy preasure build up on the enemy Champion</t>
+  </si>
+  <si>
+    <t>Column1</t>
+  </si>
+  <si>
     <t>dorans-shield</t>
   </si>
   <si>
@@ -651,6 +850,126 @@
     <t>Initial filename/ID example; Jan to confirm item facts and source.</t>
   </si>
   <si>
+    <t>Grants health and health regeneration.Taking damage from enemys restores health over time</t>
+  </si>
+  <si>
+    <t>stridebreaker</t>
+  </si>
+  <si>
+    <t>Stridebreaker</t>
+  </si>
+  <si>
+    <t>Provides attack damage, attack speed, health.Its active effect damages and slows nearby enemies</t>
+  </si>
+  <si>
+    <t>beserkers-greaves</t>
+  </si>
+  <si>
+    <t>Berserker's Greaves</t>
+  </si>
+  <si>
+    <t>Boots that provide attack speed, increasing attack frequency and improving certain champion abilities</t>
+  </si>
+  <si>
+    <t>phantom-dancer</t>
+  </si>
+  <si>
+    <t>Phantom Dancer</t>
+  </si>
+  <si>
+    <t>Provides attack speed,critical strike chance, and movement speed.Attacking enemies grants additional combat mobility</t>
+  </si>
+  <si>
+    <t>dead-mans-plate</t>
+  </si>
+  <si>
+    <t>Dead Man's Plate</t>
+  </si>
+  <si>
+    <t>Provides health and armor.Moving builds momentum, increasing movement speed and empowering your next attack</t>
+  </si>
+  <si>
+    <t>force-of-nature</t>
+  </si>
+  <si>
+    <t>Force of Nature</t>
+  </si>
+  <si>
+    <t>Provides health and magic resistance.Taking magic damage grants increased mobility and magic durability</t>
+  </si>
+  <si>
+    <t>steraks-gage</t>
+  </si>
+  <si>
+    <t>Sterak's Gage</t>
+  </si>
+  <si>
+    <t>Provides health and bonus attack damage.Taking heavy damage grants a temporary shield</t>
+  </si>
+  <si>
+    <t>scorchclaw-pup</t>
+  </si>
+  <si>
+    <t>Scorchclaw Pup</t>
+  </si>
+  <si>
+    <t>Jungle companion that helps clear camps and eventually grants a damaging burn effect against champions.</t>
+  </si>
+  <si>
+    <t>plated-steelcaps</t>
+  </si>
+  <si>
+    <t>Plated Steelcaps</t>
+  </si>
+  <si>
+    <t>Boots that provide Armor and reduce damage from enemy basic attacks.</t>
+  </si>
+  <si>
+    <t>spirit-visage</t>
+  </si>
+  <si>
+    <t>Spirit Visage</t>
+  </si>
+  <si>
+    <t>Grants Health and Magic Resistance while increasing healing received.</t>
+  </si>
+  <si>
+    <t>thornmail</t>
+  </si>
+  <si>
+    <t>Thornmail</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Grants Health and Armor. Applies Grievous Wounds to enemies that damage you.</t>
+  </si>
+  <si>
+    <t>guardian-angel</t>
+  </si>
+  <si>
+    <t>Guardian Angel</t>
+  </si>
+  <si>
+    <t>Grants Attack Damage and Armor. Revives you upon death.</t>
+  </si>
+  <si>
+    <t>dorans-blade</t>
+  </si>
+  <si>
+    <t>Doran's Blade</t>
+  </si>
+  <si>
+    <t>Grants Health, Attack Damage, and Life Steal</t>
+  </si>
+  <si>
+    <t>blade-of-the-ruined-king</t>
+  </si>
+  <si>
+    <t>Blade of the Ruined King</t>
+  </si>
+  <si>
+    <t>Grants Attack Damage, Attack Speed, and Life Steal. Attacks deal bonus damage based on enemy health</t>
+  </si>
+  <si>
     <t>IsPrimary</t>
   </si>
   <si>
@@ -666,6 +985,24 @@
     <t>Initial structural example only.</t>
   </si>
   <si>
+    <t>BUILD002</t>
+  </si>
+  <si>
+    <t>Garen Top Build</t>
+  </si>
+  <si>
+    <t>BUILD003</t>
+  </si>
+  <si>
+    <t>Warwick Jungle Build</t>
+  </si>
+  <si>
+    <t>BUILD004</t>
+  </si>
+  <si>
+    <t>Warwick Top Build</t>
+  </si>
+  <si>
     <t>Stage</t>
   </si>
   <si>
@@ -687,9 +1024,6 @@
     <t>Medium</t>
   </si>
   <si>
-    <t>No</t>
-  </si>
-  <si>
     <t>Boots</t>
   </si>
   <si>
@@ -700,6 +1034,231 @@
   </si>
   <si>
     <t>Situational</t>
+  </si>
+  <si>
+    <t>RuneId</t>
+  </si>
+  <si>
+    <t>Path</t>
+  </si>
+  <si>
+    <t>BeginnerDescription</t>
+  </si>
+  <si>
+    <t>Precision</t>
+  </si>
+  <si>
+    <t>Conqueror</t>
+  </si>
+  <si>
+    <t>Rewards champions who remain in combat and build up damage.</t>
+  </si>
+  <si>
+    <t>conqueror.webp</t>
+  </si>
+  <si>
+    <t>lethal-tempo</t>
+  </si>
+  <si>
+    <t>Lethal Tempo</t>
+  </si>
+  <si>
+    <t>Supports champions who rely on repeated basic attacks in longer fights.</t>
+  </si>
+  <si>
+    <t>lethal-tempo.webp</t>
+  </si>
+  <si>
+    <t>press-the-attack</t>
+  </si>
+  <si>
+    <t>Press the Attack</t>
+  </si>
+  <si>
+    <t>Rewards repeatedly attacking the same enemy champion.</t>
+  </si>
+  <si>
+    <t>press-the-attack.webp</t>
+  </si>
+  <si>
+    <t>fleet-footwork</t>
+  </si>
+  <si>
+    <t>Fleet Footwork</t>
+  </si>
+  <si>
+    <t>Provides sustain and mobility after moving and attacking.</t>
+  </si>
+  <si>
+    <t>fleet-footwork.webp</t>
+  </si>
+  <si>
+    <t>electrocute</t>
+  </si>
+  <si>
+    <t>Domination</t>
+  </si>
+  <si>
+    <t>Electrocute</t>
+  </si>
+  <si>
+    <t>Adds burst damage after quickly hitting an enemy with several attacks or abilities.</t>
+  </si>
+  <si>
+    <t>electrocute.webp</t>
+  </si>
+  <si>
+    <t>dark-harvest</t>
+  </si>
+  <si>
+    <t>Dark Harvest</t>
+  </si>
+  <si>
+    <t>Rewards damaging low-health enemies and collecting souls over the course of a match.</t>
+  </si>
+  <si>
+    <t>dark-harvest.webp</t>
+  </si>
+  <si>
+    <t>hail-of-blades</t>
+  </si>
+  <si>
+    <t>Hail of Blades</t>
+  </si>
+  <si>
+    <t>Provides a rapid burst of attack speed when combat begins.</t>
+  </si>
+  <si>
+    <t>hail-of-blades.webp</t>
+  </si>
+  <si>
+    <t>summon-aery</t>
+  </si>
+  <si>
+    <t>Sorcery</t>
+  </si>
+  <si>
+    <t>Summon Aery</t>
+  </si>
+  <si>
+    <t>Adds reliable damage to attacks and abilities or strengthens protection for allies.</t>
+  </si>
+  <si>
+    <t>summon-aery.webp</t>
+  </si>
+  <si>
+    <t>arcane-comet</t>
+  </si>
+  <si>
+    <t>Arcane Comet</t>
+  </si>
+  <si>
+    <t>Adds ranged damage when an ability hits an enemy champion.</t>
+  </si>
+  <si>
+    <t>arcane-comet.webp</t>
+  </si>
+  <si>
+    <t>stormraiders-surge</t>
+  </si>
+  <si>
+    <t>Stormraider's Surge</t>
+  </si>
+  <si>
+    <t>Rewards dealing substantial damage quickly with a burst of movement speed.</t>
+  </si>
+  <si>
+    <t>stormraiders-surge.webp</t>
+  </si>
+  <si>
+    <t>deathfire-touch</t>
+  </si>
+  <si>
+    <t>Deathfire Touch</t>
+  </si>
+  <si>
+    <t>Adds a damage-over-time effect to damaging attacks and abilities.</t>
+  </si>
+  <si>
+    <t>deathfire-touch.webp</t>
+  </si>
+  <si>
+    <t>aftershock</t>
+  </si>
+  <si>
+    <t>Resolve</t>
+  </si>
+  <si>
+    <t>Aftershock</t>
+  </si>
+  <si>
+    <t>Temporarily increases durability after immobilising an enemy.</t>
+  </si>
+  <si>
+    <t>aftershock.webp</t>
+  </si>
+  <si>
+    <t>grasp-of-the-undying</t>
+  </si>
+  <si>
+    <t>Grasp of the Undying</t>
+  </si>
+  <si>
+    <t>Rewards periodic attacks against enemy champions during extended lane combat.</t>
+  </si>
+  <si>
+    <t>grasp-of-the-undying.webp</t>
+  </si>
+  <si>
+    <t>guardian</t>
+  </si>
+  <si>
+    <t>Guardian</t>
+  </si>
+  <si>
+    <t>Protects nearby allies when they take damage.</t>
+  </si>
+  <si>
+    <t>guardian.webp</t>
+  </si>
+  <si>
+    <t>glacial-augment</t>
+  </si>
+  <si>
+    <t>Inspiration</t>
+  </si>
+  <si>
+    <t>Glacial Augment</t>
+  </si>
+  <si>
+    <t>Creates slowing effects after immobilising an enemy.</t>
+  </si>
+  <si>
+    <t>glacial-augment.webp</t>
+  </si>
+  <si>
+    <t>unsealed-spellbook</t>
+  </si>
+  <si>
+    <t>Unsealed Spellbook</t>
+  </si>
+  <si>
+    <t>Allows summoner spells to be exchanged during the match.</t>
+  </si>
+  <si>
+    <t>unsealed-spellbook.webp</t>
+  </si>
+  <si>
+    <t>first-strike</t>
+  </si>
+  <si>
+    <t>First Strike</t>
+  </si>
+  <si>
+    <t>Rewards initiating combat before the enemy damages you.</t>
+  </si>
+  <si>
+    <t>first-strike.webp</t>
   </si>
 </sst>
 </file>
@@ -709,7 +1268,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\-mmm\-yyyy"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -741,8 +1300,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -754,8 +1318,20 @@
         <fgColor rgb="FF1F4E78"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDCE6F1"/>
+        <bgColor rgb="FFDCE6F1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -763,12 +1339,49 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF95B3D7"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF95B3D7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF95B3D7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF95B3D7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF95B3D7"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF95B3D7"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF95B3D7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF95B3D7"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -785,12 +1398,94 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <name val="Calibri"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <name val="Calibri"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <name val="Calibri"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -838,9 +1533,9 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="tblRecommendations" displayName="tblRecommendations" ref="A1:L21">
-  <autoFilter ref="A1:L21" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
-  <tableColumns count="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="tblRecommendations" displayName="tblRecommendations" ref="A1:N21">
+  <autoFilter ref="A1:N21" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
+  <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="RecommendationId"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="ChampionId"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="LaneId"/>
@@ -850,6 +1545,8 @@
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0200-000007000000}" name="Recommended"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0200-000008000000}" name="Why"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0200-000009000000}" name="SourceUrl"/>
+    <tableColumn id="14" xr3:uid="{116F72A5-BA9F-44E0-8F97-FF17D9F0FBE4}" name="KeystoneRuneId" dataDxfId="2"/>
+    <tableColumn id="13" xr3:uid="{10F6E20F-DC5A-440C-BA33-B8425D9B9EEF}" name="RuneReason" dataDxfId="1"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0200-00000A000000}" name="ResearchNotes"/>
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0200-00000B000000}" name="ReviewedBy"/>
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0200-00000C000000}" name="LastReviewed"/>
@@ -859,11 +1556,12 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="tblItems" displayName="tblItems" ref="A1:G21">
-  <autoFilter ref="A1:G21" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
-  <tableColumns count="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{00000000-000C-0000-FFFF-FFFF03000000}" name="tblItems" displayName="tblItems" ref="A1:H21">
+  <autoFilter ref="A1:H21" xr:uid="{00000000-0009-0000-0100-000004000000}"/>
+  <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0300-000001000000}" name="ItemId"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0300-000002000000}" name="Name"/>
+    <tableColumn id="8" xr3:uid="{4B3324A3-B21B-4FD1-8462-C97A03DD9C91}" name="Column1" dataDxfId="0"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0300-000003000000}" name="Description"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0300-000004000000}" name="ImageFileName"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0300-000005000000}" name="SourceUrl"/>
@@ -892,8 +1590,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="tblBuildItems" displayName="tblBuildItems" ref="A1:E21">
-  <autoFilter ref="A1:E21" xr:uid="{00000000-0009-0000-0100-000006000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="tblBuildItems" displayName="tblBuildItems" ref="A1:E23">
+  <autoFilter ref="A1:E23" xr:uid="{00000000-0009-0000-0100-000006000000}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="BuildId"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="ItemId"/>
@@ -1502,7 +2200,7 @@
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="3" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>70</v>
@@ -1548,7 +2246,7 @@
       </c>
       <c r="C8" s="3"/>
       <c r="D8" s="3" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>80</v>
@@ -1564,158 +2262,254 @@
     </row>
     <row r="9" spans="1:9" ht="30.75">
       <c r="A9" s="3" t="s">
-        <v>83</v>
+        <v>46</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>84</v>
+        <v>47</v>
       </c>
       <c r="C9" s="3"/>
       <c r="D9" s="3" t="s">
         <v>49</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>85</v>
+        <v>50</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>86</v>
+        <v>51</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>87</v>
+        <v>52</v>
       </c>
       <c r="H9" s="3"/>
       <c r="I9" s="4"/>
     </row>
     <row r="10" spans="1:9" ht="30.75">
       <c r="A10" s="3" t="s">
-        <v>88</v>
+        <v>57</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>89</v>
+        <v>58</v>
       </c>
       <c r="C10" s="3"/>
       <c r="D10" s="3" t="s">
         <v>49</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="H10" s="3"/>
       <c r="I10" s="4"/>
     </row>
     <row r="11" spans="1:9" ht="30.75">
       <c r="A11" s="3" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="3" t="s">
         <v>49</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="H11" s="3"/>
       <c r="I11" s="4"/>
     </row>
-    <row r="12" spans="1:9">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
+    <row r="12" spans="1:9" ht="30.75">
+      <c r="A12" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>91</v>
+      </c>
       <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
+      <c r="D12" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>94</v>
+      </c>
       <c r="H12" s="3"/>
       <c r="I12" s="4"/>
     </row>
-    <row r="13" spans="1:9">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
+    <row r="13" spans="1:9" ht="30.75">
+      <c r="A13" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>96</v>
+      </c>
       <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
+      <c r="D13" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="H13" s="3"/>
       <c r="I13" s="4"/>
     </row>
-    <row r="14" spans="1:9">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
+    <row r="14" spans="1:9" ht="30.75">
+      <c r="A14" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>101</v>
+      </c>
       <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
+      <c r="D14" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>104</v>
+      </c>
       <c r="H14" s="3"/>
       <c r="I14" s="4"/>
     </row>
-    <row r="15" spans="1:9">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
+    <row r="15" spans="1:9" ht="30.75">
+      <c r="A15" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>55</v>
+      </c>
       <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
+      <c r="D15" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>107</v>
+      </c>
       <c r="H15" s="3"/>
       <c r="I15" s="4"/>
     </row>
-    <row r="16" spans="1:9">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3"/>
+    <row r="16" spans="1:9" ht="45.75">
+      <c r="A16" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>109</v>
+      </c>
       <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
+      <c r="D16" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>112</v>
+      </c>
       <c r="H16" s="3"/>
       <c r="I16" s="4"/>
     </row>
-    <row r="17" spans="1:9">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
+    <row r="17" spans="1:9" ht="30.75">
+      <c r="A17" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>114</v>
+      </c>
       <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
+      <c r="D17" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>117</v>
+      </c>
       <c r="H17" s="3"/>
       <c r="I17" s="4"/>
     </row>
-    <row r="18" spans="1:9">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
+    <row r="18" spans="1:9" ht="45.75">
+      <c r="A18" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>119</v>
+      </c>
       <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
+      <c r="D18" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>122</v>
+      </c>
       <c r="H18" s="3"/>
       <c r="I18" s="4"/>
     </row>
-    <row r="19" spans="1:9">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
+    <row r="19" spans="1:9" ht="30.75">
+      <c r="A19" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>124</v>
+      </c>
       <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
+      <c r="D19" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="G19" s="5" t="s">
+        <v>127</v>
+      </c>
       <c r="H19" s="3"/>
       <c r="I19" s="4"/>
     </row>
@@ -1724,17 +2518,25 @@
     <hyperlink ref="G5" r:id="rId1" xr:uid="{4221F828-001F-468E-9E75-CB7D63B6BA78}"/>
     <hyperlink ref="G6" r:id="rId2" xr:uid="{762397C8-1CD1-45BB-BD11-365F1A91F1F5}"/>
     <hyperlink ref="G7" r:id="rId3" xr:uid="{A7CB9255-672A-469B-B387-C5EFF7CD6880}"/>
-    <hyperlink ref="G9" r:id="rId4" xr:uid="{14FCFC72-1526-4159-BDB9-2DEC6BCB29E9}"/>
-    <hyperlink ref="G10" r:id="rId5" xr:uid="{B8BEF309-A3A2-46E1-95AF-7D18A3AEE31C}"/>
-    <hyperlink ref="G11" r:id="rId6" xr:uid="{AA8B2E10-1788-41CB-B862-F3FCB95F51D9}"/>
+    <hyperlink ref="G11" r:id="rId4" xr:uid="{14FCFC72-1526-4159-BDB9-2DEC6BCB29E9}"/>
+    <hyperlink ref="G12" r:id="rId5" xr:uid="{B8BEF309-A3A2-46E1-95AF-7D18A3AEE31C}"/>
+    <hyperlink ref="G13" r:id="rId6" xr:uid="{AA8B2E10-1788-41CB-B862-F3FCB95F51D9}"/>
     <hyperlink ref="G8" r:id="rId7" xr:uid="{1EB11F8C-1845-4368-BE3A-6397F34E89DC}"/>
     <hyperlink ref="G2" r:id="rId8" xr:uid="{1F476FB8-2F65-4E31-8806-2934A4D4AFF6}"/>
     <hyperlink ref="G4" r:id="rId9" xr:uid="{5E220BED-EFE0-434F-AC54-538856FA6AC1}"/>
+    <hyperlink ref="G9" r:id="rId10" xr:uid="{40DE9256-4B6C-4A28-B1B8-E46CC9DEA8C1}"/>
+    <hyperlink ref="G10" r:id="rId11" xr:uid="{66A55C05-251C-4D30-8FA2-9BA68BC9D003}"/>
+    <hyperlink ref="G14" r:id="rId12" xr:uid="{CC017235-9635-4D45-884A-5937C10F4564}"/>
+    <hyperlink ref="G15" r:id="rId13" xr:uid="{7B4A2518-A4FF-4FB6-ABC0-6710E2D4AA4C}"/>
+    <hyperlink ref="G16" r:id="rId14" xr:uid="{071C59B2-5D86-4F6A-B33C-778CE56AD474}"/>
+    <hyperlink ref="G17" r:id="rId15" xr:uid="{15FB2263-4E8B-4387-8059-41B5699DD65E}"/>
+    <hyperlink ref="G18" r:id="rId16" xr:uid="{FA6BE657-6157-4F1A-BC8D-7F0AA899B7B8}"/>
+    <hyperlink ref="G19" r:id="rId17" xr:uid="{0B2E789A-DD8A-41AA-87E4-02A3D9943F68}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing r:id="rId10"/>
+  <legacyDrawing r:id="rId18"/>
   <tableParts count="1">
-    <tablePart r:id="rId11"/>
+    <tablePart r:id="rId19"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1760,13 +2562,13 @@
         <v>38</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>98</v>
+        <v>128</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>41</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>99</v>
+        <v>129</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>42</v>
@@ -1777,106 +2579,106 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="2" t="s">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>101</v>
+        <v>131</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>102</v>
+        <v>132</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>103</v>
+        <v>133</v>
       </c>
       <c r="E2" s="2">
         <v>1</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>104</v>
+        <v>134</v>
       </c>
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="2" t="s">
-        <v>105</v>
+        <v>135</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>106</v>
+        <v>136</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>106</v>
+        <v>136</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>107</v>
+        <v>137</v>
       </c>
       <c r="E3" s="2">
         <v>2</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>108</v>
+        <v>138</v>
       </c>
       <c r="G3" s="2"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="2" t="s">
-        <v>109</v>
+        <v>139</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>110</v>
+        <v>140</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>111</v>
+        <v>141</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>112</v>
+        <v>142</v>
       </c>
       <c r="E4" s="2">
         <v>3</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>113</v>
+        <v>143</v>
       </c>
       <c r="G4" s="2"/>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="2" t="s">
-        <v>114</v>
+        <v>144</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>114</v>
+        <v>144</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>115</v>
+        <v>145</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>116</v>
+        <v>146</v>
       </c>
       <c r="E5" s="2">
         <v>4</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>117</v>
+        <v>147</v>
       </c>
       <c r="G5" s="2"/>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="2" t="s">
-        <v>118</v>
+        <v>148</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>119</v>
+        <v>149</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>119</v>
+        <v>149</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="E6" s="2">
         <v>5</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>121</v>
+        <v>151</v>
       </c>
       <c r="G6" s="2"/>
     </row>
@@ -1891,7 +2693,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -1902,13 +2704,13 @@
     <col min="6" max="6" width="24" customWidth="1"/>
     <col min="7" max="7" width="15" customWidth="1"/>
     <col min="8" max="8" width="60" customWidth="1"/>
-    <col min="9" max="9" width="42" customWidth="1"/>
-    <col min="10" max="10" width="45" customWidth="1"/>
-    <col min="11" max="11" width="20" customWidth="1"/>
-    <col min="12" max="12" width="16" customWidth="1"/>
+    <col min="9" max="11" width="42" customWidth="1"/>
+    <col min="12" max="12" width="45" customWidth="1"/>
+    <col min="13" max="13" width="20" customWidth="1"/>
+    <col min="14" max="14" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="24" customHeight="1">
+    <row r="1" spans="1:14" ht="24" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>32</v>
       </c>
@@ -1919,42 +2721,48 @@
         <v>28</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>122</v>
+        <v>152</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>123</v>
+        <v>153</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>124</v>
+        <v>154</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>125</v>
+        <v>155</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>43</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="N1" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="30.75">
+    <row r="2" spans="1:14" ht="30.75">
       <c r="A2" s="2" t="s">
-        <v>127</v>
+        <v>159</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>46</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>100</v>
+        <v>130</v>
       </c>
       <c r="D2" s="3">
         <v>5</v>
@@ -1963,30 +2771,32 @@
         <v>49</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>128</v>
+        <v>160</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>129</v>
+        <v>161</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>130</v>
+        <v>162</v>
       </c>
       <c r="I2" s="3"/>
-      <c r="J2" s="3" t="s">
-        <v>131</v>
-      </c>
+      <c r="J2" s="3"/>
       <c r="K2" s="3"/>
-      <c r="L2" s="4"/>
-    </row>
-    <row r="3" spans="1:12">
+      <c r="L2" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="M2" s="3"/>
+      <c r="N2" s="4"/>
+    </row>
+    <row r="3" spans="1:14">
       <c r="A3" s="3" t="s">
-        <v>132</v>
+        <v>164</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>63</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>118</v>
+        <v>148</v>
       </c>
       <c r="D3" s="3">
         <v>5</v>
@@ -1995,276 +2805,528 @@
         <v>49</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>133</v>
+        <v>165</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>129</v>
+        <v>161</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>130</v>
+        <v>162</v>
       </c>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
-      <c r="L3" s="4"/>
-    </row>
-    <row r="4" spans="1:12">
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="4"/>
+    </row>
+    <row r="4" spans="1:14">
       <c r="A4" s="3" t="s">
-        <v>134</v>
+        <v>166</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>68</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>118</v>
+        <v>148</v>
       </c>
       <c r="D4" s="3">
         <v>4</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>49</v>
+        <v>167</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>135</v>
+        <v>168</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>129</v>
+        <v>161</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>136</v>
+        <v>169</v>
       </c>
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
-      <c r="L4" s="4"/>
-    </row>
-    <row r="5" spans="1:12">
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="4"/>
+    </row>
+    <row r="5" spans="1:14">
       <c r="A5" s="3" t="s">
-        <v>137</v>
+        <v>170</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>73</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>118</v>
+        <v>148</v>
       </c>
       <c r="D5" s="3">
         <v>4</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>138</v>
+        <v>167</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>139</v>
+        <v>171</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>129</v>
+        <v>161</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>140</v>
+        <v>172</v>
       </c>
       <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
+      <c r="J5" s="3" t="s">
+        <v>173</v>
+      </c>
       <c r="K5" s="3"/>
-      <c r="L5" s="4"/>
-    </row>
-    <row r="6" spans="1:12">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
+      <c r="N5" s="4"/>
+    </row>
+    <row r="6" spans="1:14">
+      <c r="A6" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="D6" s="3">
+        <v>4</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>176</v>
+      </c>
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
       <c r="K6" s="3"/>
-      <c r="L6" s="4"/>
-    </row>
-    <row r="7" spans="1:12">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
+      <c r="L6" s="3"/>
+      <c r="M6" s="3"/>
+      <c r="N6" s="4"/>
+    </row>
+    <row r="7" spans="1:14">
+      <c r="A7" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="D7" s="3">
+        <v>5</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>178</v>
+      </c>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
-      <c r="L7" s="4"/>
-    </row>
-    <row r="8" spans="1:12">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
+      <c r="L7" s="3"/>
+      <c r="M7" s="3"/>
+      <c r="N7" s="4"/>
+    </row>
+    <row r="8" spans="1:14">
+      <c r="A8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="D8" s="3">
+        <v>5</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>180</v>
+      </c>
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
-      <c r="L8" s="4"/>
-    </row>
-    <row r="9" spans="1:12">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="3"/>
+      <c r="N8" s="4"/>
+    </row>
+    <row r="9" spans="1:14">
+      <c r="A9" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="D9" s="3">
+        <v>5</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>183</v>
+      </c>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
-      <c r="L9" s="4"/>
-    </row>
-    <row r="10" spans="1:12">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
+      <c r="L9" s="3"/>
+      <c r="M9" s="3"/>
+      <c r="N9" s="4"/>
+    </row>
+    <row r="10" spans="1:14">
+      <c r="A10" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="D10" s="3">
+        <v>5</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>185</v>
+      </c>
       <c r="I10" s="3"/>
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
-      <c r="L10" s="4"/>
-    </row>
-    <row r="11" spans="1:12">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
+      <c r="L10" s="3"/>
+      <c r="M10" s="3"/>
+      <c r="N10" s="4"/>
+    </row>
+    <row r="11" spans="1:14">
+      <c r="A11" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="D11" s="3">
+        <v>4</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>187</v>
+      </c>
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
-      <c r="L11" s="4"/>
-    </row>
-    <row r="12" spans="1:12">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
+      <c r="L11" s="3"/>
+      <c r="M11" s="3"/>
+      <c r="N11" s="4"/>
+    </row>
+    <row r="12" spans="1:14">
+      <c r="A12" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="D12" s="3">
+        <v>5</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>190</v>
+      </c>
       <c r="I12" s="3"/>
       <c r="J12" s="3"/>
       <c r="K12" s="3"/>
-      <c r="L12" s="4"/>
-    </row>
-    <row r="13" spans="1:12">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
+      <c r="L12" s="3"/>
+      <c r="M12" s="3"/>
+      <c r="N12" s="4"/>
+    </row>
+    <row r="13" spans="1:14">
+      <c r="A13" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="D13" s="3">
+        <v>4</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>192</v>
+      </c>
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
-      <c r="L13" s="4"/>
-    </row>
-    <row r="14" spans="1:12">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
+      <c r="L13" s="3"/>
+      <c r="M13" s="3"/>
+      <c r="N13" s="4"/>
+    </row>
+    <row r="14" spans="1:14">
+      <c r="A14" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="D14" s="3">
+        <v>4</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>194</v>
+      </c>
       <c r="I14" s="3"/>
       <c r="J14" s="3"/>
       <c r="K14" s="3"/>
-      <c r="L14" s="4"/>
-    </row>
-    <row r="15" spans="1:12">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
+      <c r="L14" s="3"/>
+      <c r="M14" s="3"/>
+      <c r="N14" s="4"/>
+    </row>
+    <row r="15" spans="1:14">
+      <c r="A15" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="D15" s="3">
+        <v>5</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>197</v>
+      </c>
       <c r="I15" s="3"/>
       <c r="J15" s="3"/>
       <c r="K15" s="3"/>
-      <c r="L15" s="4"/>
-    </row>
-    <row r="16" spans="1:12">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
-      <c r="H16" s="3"/>
+      <c r="L15" s="3"/>
+      <c r="M15" s="3"/>
+      <c r="N15" s="4"/>
+    </row>
+    <row r="16" spans="1:14">
+      <c r="A16" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="D16" s="3">
+        <v>5</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>199</v>
+      </c>
       <c r="I16" s="3"/>
       <c r="J16" s="3"/>
       <c r="K16" s="3"/>
-      <c r="L16" s="4"/>
-    </row>
-    <row r="17" spans="1:12">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
+      <c r="L16" s="3"/>
+      <c r="M16" s="3"/>
+      <c r="N16" s="4"/>
+    </row>
+    <row r="17" spans="1:14">
+      <c r="A17" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="D17" s="3">
+        <v>4</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>201</v>
+      </c>
       <c r="I17" s="3"/>
       <c r="J17" s="3"/>
       <c r="K17" s="3"/>
-      <c r="L17" s="4"/>
-    </row>
-    <row r="18" spans="1:12">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
+      <c r="L17" s="3"/>
+      <c r="M17" s="3"/>
+      <c r="N17" s="4"/>
+    </row>
+    <row r="18" spans="1:14">
+      <c r="A18" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>139</v>
+      </c>
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
+      <c r="G18" s="3" t="s">
+        <v>203</v>
+      </c>
       <c r="H18" s="3"/>
       <c r="I18" s="3"/>
       <c r="J18" s="3"/>
       <c r="K18" s="3"/>
-      <c r="L18" s="4"/>
-    </row>
-    <row r="19" spans="1:12">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
+      <c r="L18" s="3"/>
+      <c r="M18" s="3"/>
+      <c r="N18" s="4"/>
+    </row>
+    <row r="19" spans="1:14" ht="30.75">
+      <c r="A19" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="D19" s="3">
+        <v>5</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>205</v>
+      </c>
       <c r="I19" s="3"/>
       <c r="J19" s="3"/>
       <c r="K19" s="3"/>
-      <c r="L19" s="4"/>
-    </row>
-    <row r="20" spans="1:12">
+      <c r="L19" s="3"/>
+      <c r="M19" s="3"/>
+      <c r="N19" s="4"/>
+    </row>
+    <row r="20" spans="1:14">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -2276,9 +3338,11 @@
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
       <c r="K20" s="3"/>
-      <c r="L20" s="4"/>
-    </row>
-    <row r="21" spans="1:12">
+      <c r="L20" s="3"/>
+      <c r="M20" s="3"/>
+      <c r="N20" s="4"/>
+    </row>
+    <row r="21" spans="1:14">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
@@ -2290,7 +3354,9 @@
       <c r="I21" s="3"/>
       <c r="J21" s="3"/>
       <c r="K21" s="3"/>
-      <c r="L21" s="4"/>
+      <c r="L21" s="3"/>
+      <c r="M21" s="3"/>
+      <c r="N21" s="4"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="D2:D500">
@@ -2315,19 +3381,19 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="55" customWidth="1"/>
-    <col min="4" max="4" width="30" customWidth="1"/>
-    <col min="5" max="5" width="42" customWidth="1"/>
-    <col min="6" max="6" width="45" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="2" max="3" width="28" customWidth="1"/>
+    <col min="4" max="4" width="55" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
+    <col min="6" max="6" width="42" customWidth="1"/>
+    <col min="7" max="7" width="45" customWidth="1"/>
+    <col min="8" max="8" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="24" customHeight="1">
+    <row r="1" spans="1:8" ht="24" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>30</v>
       </c>
@@ -2335,208 +3401,315 @@
         <v>38</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="30.75">
+    <row r="2" spans="1:8" ht="30.75">
       <c r="A2" s="2" t="s">
-        <v>141</v>
+        <v>207</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="C2" s="3"/>
-      <c r="D2" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="G2" s="4"/>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
+        <v>208</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="H2" s="4"/>
+    </row>
+    <row r="3" spans="1:8" ht="30.75">
+      <c r="A3" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>208</v>
+      </c>
       <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
+      <c r="D3" s="3" t="s">
+        <v>211</v>
+      </c>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
-      <c r="G3" s="4"/>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="4"/>
+    </row>
+    <row r="4" spans="1:8" ht="30.75">
+      <c r="A4" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>213</v>
+      </c>
       <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
+      <c r="D4" s="3" t="s">
+        <v>214</v>
+      </c>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
-      <c r="G4" s="4"/>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="4"/>
+    </row>
+    <row r="5" spans="1:8" ht="30.75">
+      <c r="A5" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>216</v>
+      </c>
       <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
+      <c r="D5" s="3" t="s">
+        <v>217</v>
+      </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
-      <c r="G5" s="4"/>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="4"/>
+    </row>
+    <row r="6" spans="1:8" ht="30.75">
+      <c r="A6" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>219</v>
+      </c>
       <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
+      <c r="D6" s="3" t="s">
+        <v>220</v>
+      </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
-      <c r="G6" s="4"/>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="4"/>
+    </row>
+    <row r="7" spans="1:8" ht="30.75">
+      <c r="A7" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>222</v>
+      </c>
       <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
+      <c r="D7" s="3" t="s">
+        <v>223</v>
+      </c>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
-      <c r="G7" s="4"/>
-    </row>
-    <row r="8" spans="1:7">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="4"/>
+    </row>
+    <row r="8" spans="1:8" ht="30.75">
+      <c r="A8" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>225</v>
+      </c>
       <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
+      <c r="D8" s="3" t="s">
+        <v>226</v>
+      </c>
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
-      <c r="G8" s="4"/>
-    </row>
-    <row r="9" spans="1:7">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="4"/>
+    </row>
+    <row r="9" spans="1:8" ht="30.75">
+      <c r="A9" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>228</v>
+      </c>
       <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
+      <c r="D9" s="3" t="s">
+        <v>229</v>
+      </c>
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
-      <c r="G9" s="4"/>
-    </row>
-    <row r="10" spans="1:7">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="4"/>
+    </row>
+    <row r="10" spans="1:8" ht="30.75">
+      <c r="A10" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>231</v>
+      </c>
       <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
+      <c r="D10" s="3" t="s">
+        <v>232</v>
+      </c>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
-      <c r="G10" s="4"/>
-    </row>
-    <row r="11" spans="1:7">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="4"/>
+    </row>
+    <row r="11" spans="1:8" ht="30.75">
+      <c r="A11" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>234</v>
+      </c>
       <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
+      <c r="D11" s="3" t="s">
+        <v>235</v>
+      </c>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
-      <c r="G11" s="4"/>
-    </row>
-    <row r="12" spans="1:7">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="4"/>
+    </row>
+    <row r="12" spans="1:8" ht="30.75">
+      <c r="A12" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>237</v>
+      </c>
       <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
+      <c r="D12" s="3" t="s">
+        <v>238</v>
+      </c>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
-      <c r="G12" s="4"/>
-    </row>
-    <row r="13" spans="1:7">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="4"/>
+    </row>
+    <row r="13" spans="1:8" ht="30.75">
+      <c r="A13" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>240</v>
+      </c>
       <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
+      <c r="D13" s="3" t="s">
+        <v>241</v>
+      </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
-      <c r="G13" s="4"/>
-    </row>
-    <row r="14" spans="1:7">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="4"/>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>243</v>
+      </c>
       <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
+      <c r="D14" s="3" t="s">
+        <v>244</v>
+      </c>
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
-      <c r="G14" s="4"/>
-    </row>
-    <row r="15" spans="1:7">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="4"/>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>246</v>
+      </c>
       <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
+      <c r="D15" s="3" t="s">
+        <v>247</v>
+      </c>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
-      <c r="G15" s="4"/>
-    </row>
-    <row r="16" spans="1:7">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="4"/>
+    </row>
+    <row r="16" spans="1:8" ht="30.75">
+      <c r="A16" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>249</v>
+      </c>
       <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
+      <c r="D16" s="3" t="s">
+        <v>250</v>
+      </c>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
-      <c r="G16" s="4"/>
-    </row>
-    <row r="17" spans="1:7">
+      <c r="G16" s="3"/>
+      <c r="H16" s="4"/>
+    </row>
+    <row r="17" spans="1:8">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
-      <c r="G17" s="4"/>
-    </row>
-    <row r="18" spans="1:7">
+      <c r="G17" s="3"/>
+      <c r="H17" s="4"/>
+    </row>
+    <row r="18" spans="1:8">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
-      <c r="G18" s="4"/>
-    </row>
-    <row r="19" spans="1:7">
+      <c r="G18" s="3"/>
+      <c r="H18" s="4"/>
+    </row>
+    <row r="19" spans="1:8">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
-      <c r="G19" s="4"/>
-    </row>
-    <row r="20" spans="1:7">
+      <c r="G19" s="3"/>
+      <c r="H19" s="4"/>
+    </row>
+    <row r="20" spans="1:8">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
-      <c r="G20" s="4"/>
-    </row>
-    <row r="21" spans="1:7">
+      <c r="G20" s="3"/>
+      <c r="H20" s="4"/>
+    </row>
+    <row r="21" spans="1:8">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
-      <c r="G21" s="4"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2576,7 +3749,7 @@
         <v>41</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>145</v>
+        <v>251</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>43</v>
@@ -2590,30 +3763,36 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="2" t="s">
-        <v>146</v>
+        <v>252</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>127</v>
+        <v>159</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>147</v>
+        <v>253</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>148</v>
+        <v>254</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>129</v>
+        <v>161</v>
       </c>
       <c r="F2" s="3"/>
       <c r="G2" s="3" t="s">
-        <v>149</v>
+        <v>255</v>
       </c>
       <c r="H2" s="4"/>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
+      <c r="A3" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>257</v>
+      </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
@@ -2621,9 +3800,15 @@
       <c r="H3" s="4"/>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
+      <c r="A4" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>259</v>
+      </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
@@ -2631,9 +3816,15 @@
       <c r="H4" s="4"/>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
+      <c r="A5" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>261</v>
+      </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
@@ -2811,7 +4002,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="3" width="18" customWidth="1"/>
@@ -2827,164 +4018,300 @@
         <v>30</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>150</v>
+        <v>262</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>99</v>
+        <v>129</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>151</v>
+        <v>263</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
-        <v>146</v>
+        <v>252</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>141</v>
+        <v>207</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>152</v>
+        <v>264</v>
       </c>
       <c r="D2" s="3">
         <v>1</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>153</v>
+        <v>265</v>
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
+      <c r="A3" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>207</v>
+      </c>
       <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
+      <c r="D3" s="3">
+        <v>1</v>
+      </c>
       <c r="E3" s="3"/>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
+      <c r="A4" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>212</v>
+      </c>
       <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
+      <c r="D4" s="3">
+        <v>2</v>
+      </c>
       <c r="E4" s="3"/>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
+      <c r="A5" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>215</v>
+      </c>
       <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
+      <c r="D5" s="3">
+        <v>3</v>
+      </c>
       <c r="E5" s="3"/>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="3"/>
-      <c r="B6" s="3"/>
+      <c r="A6" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>218</v>
+      </c>
       <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
+      <c r="D6" s="3">
+        <v>4</v>
+      </c>
       <c r="E6" s="3"/>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="3"/>
-      <c r="B7" s="3"/>
+      <c r="A7" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>221</v>
+      </c>
       <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
+      <c r="D7" s="3">
+        <v>5</v>
+      </c>
       <c r="E7" s="3"/>
     </row>
     <row r="8" spans="1:5">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
+      <c r="A8" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>224</v>
+      </c>
       <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
+      <c r="D8" s="3">
+        <v>6</v>
+      </c>
       <c r="E8" s="3"/>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
+      <c r="A9" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>227</v>
+      </c>
       <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
+      <c r="D9" s="3">
+        <v>7</v>
+      </c>
       <c r="E9" s="3"/>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
+      <c r="A10" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>230</v>
+      </c>
       <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
+      <c r="D10" s="3">
+        <v>1</v>
+      </c>
       <c r="E10" s="3"/>
     </row>
     <row r="11" spans="1:5">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
+      <c r="A11" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>212</v>
+      </c>
       <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
+      <c r="D11" s="3">
+        <v>2</v>
+      </c>
       <c r="E11" s="3"/>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
+      <c r="A12" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>233</v>
+      </c>
       <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
+      <c r="D12" s="3">
+        <v>3</v>
+      </c>
       <c r="E12" s="3"/>
     </row>
     <row r="13" spans="1:5">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
+      <c r="A13" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>236</v>
+      </c>
       <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
+      <c r="D13" s="3">
+        <v>4</v>
+      </c>
       <c r="E13" s="3"/>
     </row>
     <row r="14" spans="1:5">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
+      <c r="A14" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>239</v>
+      </c>
       <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
+      <c r="D14" s="3">
+        <v>5</v>
+      </c>
       <c r="E14" s="3"/>
     </row>
     <row r="15" spans="1:5">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
+      <c r="A15" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>227</v>
+      </c>
       <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
+      <c r="D15" s="3">
+        <v>6</v>
+      </c>
       <c r="E15" s="3"/>
     </row>
     <row r="16" spans="1:5">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3"/>
+      <c r="A16" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>242</v>
+      </c>
       <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
+      <c r="D16" s="3">
+        <v>7</v>
+      </c>
       <c r="E16" s="3"/>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
+      <c r="A17" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>245</v>
+      </c>
       <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
+      <c r="D17" s="3">
+        <v>1</v>
+      </c>
       <c r="E17" s="3"/>
     </row>
-    <row r="18" spans="1:5">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
+    <row r="18" spans="1:5" ht="30.75">
+      <c r="A18" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>248</v>
+      </c>
       <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
+      <c r="D18" s="3">
+        <v>2</v>
+      </c>
       <c r="E18" s="3"/>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
+      <c r="A19" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>233</v>
+      </c>
       <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
+      <c r="D19" s="3">
+        <v>3</v>
+      </c>
       <c r="E19" s="3"/>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
+      <c r="A20" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>212</v>
+      </c>
       <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
+      <c r="D20" s="3">
+        <v>4</v>
+      </c>
       <c r="E20" s="3"/>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
+      <c r="A21" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>236</v>
+      </c>
       <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
+      <c r="D21" s="3">
+        <v>5</v>
+      </c>
       <c r="E21" s="3"/>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="D22" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="D23" s="3">
+        <v>7</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3009,13 +4336,13 @@
         <v>40</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>154</v>
+        <v>266</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>155</v>
+        <v>267</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>122</v>
+        <v>152</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -3023,10 +4350,10 @@
         <v>49</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>129</v>
+        <v>161</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>152</v>
+        <v>264</v>
       </c>
       <c r="D2" s="2">
         <v>1</v>
@@ -3034,13 +4361,13 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
-        <v>156</v>
+        <v>268</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>157</v>
+        <v>203</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>158</v>
+        <v>269</v>
       </c>
       <c r="D3" s="2">
         <v>2</v>
@@ -3048,11 +4375,11 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="2" t="s">
-        <v>159</v>
+        <v>270</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
-        <v>160</v>
+        <v>271</v>
       </c>
       <c r="D4" s="2">
         <v>3</v>
@@ -3062,7 +4389,7 @@
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2" t="s">
-        <v>161</v>
+        <v>272</v>
       </c>
       <c r="D5" s="2">
         <v>4</v>
@@ -3079,4 +4406,419 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{841C4449-EA12-4163-BFFB-E074DBC33876}">
+  <dimension ref="A1:H18"/>
+  <sheetFormatPr defaultColWidth="49.7109375" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="30.75">
+      <c r="A1" s="12" t="s">
+        <v>273</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>274</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>275</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="F1" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="G1" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="H1" s="14" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="30.75">
+      <c r="A2" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>277</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>278</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>279</v>
+      </c>
+      <c r="F2" s="7">
+        <v>1</v>
+      </c>
+      <c r="G2" s="7"/>
+      <c r="H2" s="8"/>
+    </row>
+    <row r="3" spans="1:8" ht="45.75">
+      <c r="A3" s="9" t="s">
+        <v>280</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>276</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>281</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>282</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>283</v>
+      </c>
+      <c r="F3" s="10">
+        <v>2</v>
+      </c>
+      <c r="G3" s="10"/>
+      <c r="H3" s="11"/>
+    </row>
+    <row r="4" spans="1:8" ht="30.75">
+      <c r="A4" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>276</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>286</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="F4" s="7">
+        <v>3</v>
+      </c>
+      <c r="G4" s="7"/>
+      <c r="H4" s="8"/>
+    </row>
+    <row r="5" spans="1:8" ht="30.75">
+      <c r="A5" s="9" t="s">
+        <v>288</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>276</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>289</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>290</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>291</v>
+      </c>
+      <c r="F5" s="10">
+        <v>4</v>
+      </c>
+      <c r="G5" s="10"/>
+      <c r="H5" s="11"/>
+    </row>
+    <row r="6" spans="1:8" ht="45.75">
+      <c r="A6" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>293</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>294</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>295</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>296</v>
+      </c>
+      <c r="F6" s="7">
+        <v>1</v>
+      </c>
+      <c r="G6" s="7"/>
+      <c r="H6" s="8"/>
+    </row>
+    <row r="7" spans="1:8" ht="45.75">
+      <c r="A7" s="9" t="s">
+        <v>297</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>293</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>298</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>299</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>300</v>
+      </c>
+      <c r="F7" s="10">
+        <v>2</v>
+      </c>
+      <c r="G7" s="10"/>
+      <c r="H7" s="11"/>
+    </row>
+    <row r="8" spans="1:8" ht="30.75">
+      <c r="A8" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>293</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>303</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>304</v>
+      </c>
+      <c r="F8" s="7">
+        <v>3</v>
+      </c>
+      <c r="G8" s="7"/>
+      <c r="H8" s="8"/>
+    </row>
+    <row r="9" spans="1:8" ht="45.75">
+      <c r="A9" s="9" t="s">
+        <v>305</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>306</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>307</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>308</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>309</v>
+      </c>
+      <c r="F9" s="10">
+        <v>1</v>
+      </c>
+      <c r="G9" s="10"/>
+      <c r="H9" s="11"/>
+    </row>
+    <row r="10" spans="1:8" ht="30.75">
+      <c r="A10" s="6" t="s">
+        <v>310</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>306</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>311</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>312</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>313</v>
+      </c>
+      <c r="F10" s="7">
+        <v>2</v>
+      </c>
+      <c r="G10" s="7"/>
+      <c r="H10" s="8"/>
+    </row>
+    <row r="11" spans="1:8" ht="45.75">
+      <c r="A11" s="9" t="s">
+        <v>314</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>306</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>315</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>316</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>317</v>
+      </c>
+      <c r="F11" s="10">
+        <v>3</v>
+      </c>
+      <c r="G11" s="10"/>
+      <c r="H11" s="11"/>
+    </row>
+    <row r="12" spans="1:8" ht="30.75">
+      <c r="A12" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>306</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>321</v>
+      </c>
+      <c r="F12" s="7">
+        <v>4</v>
+      </c>
+      <c r="G12" s="7"/>
+      <c r="H12" s="8"/>
+    </row>
+    <row r="13" spans="1:8" ht="30.75">
+      <c r="A13" s="9" t="s">
+        <v>322</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>323</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>324</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>325</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>326</v>
+      </c>
+      <c r="F13" s="10">
+        <v>1</v>
+      </c>
+      <c r="G13" s="10"/>
+      <c r="H13" s="11"/>
+    </row>
+    <row r="14" spans="1:8" ht="45.75">
+      <c r="A14" s="6" t="s">
+        <v>327</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>323</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>329</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>330</v>
+      </c>
+      <c r="F14" s="7">
+        <v>2</v>
+      </c>
+      <c r="G14" s="7"/>
+      <c r="H14" s="8"/>
+    </row>
+    <row r="15" spans="1:8" ht="30.75">
+      <c r="A15" s="9" t="s">
+        <v>331</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>323</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>332</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>333</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>334</v>
+      </c>
+      <c r="F15" s="10">
+        <v>3</v>
+      </c>
+      <c r="G15" s="10"/>
+      <c r="H15" s="11"/>
+    </row>
+    <row r="16" spans="1:8" ht="30.75">
+      <c r="A16" s="6" t="s">
+        <v>335</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>336</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>337</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>338</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="F16" s="7">
+        <v>1</v>
+      </c>
+      <c r="G16" s="7"/>
+      <c r="H16" s="8"/>
+    </row>
+    <row r="17" spans="1:8" ht="30.75">
+      <c r="A17" s="9" t="s">
+        <v>340</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>336</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>341</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>342</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>343</v>
+      </c>
+      <c r="F17" s="10">
+        <v>2</v>
+      </c>
+      <c r="G17" s="10"/>
+      <c r="H17" s="11"/>
+    </row>
+    <row r="18" spans="1:8" ht="30.75">
+      <c r="A18" s="6" t="s">
+        <v>344</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>336</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>346</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="F18" s="7">
+        <v>3</v>
+      </c>
+      <c r="G18" s="7"/>
+      <c r="H18" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Spreedsheets Updated to the newest version
</commit_message>
<xml_diff>
--- a/data/league-new-player-data-template-populated.xlsx
+++ b/data/league-new-player-data-template-populated.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="531" documentId="11_91E030B3067DB12A649EB0356813936805D8A028" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E744ABE-3E4F-40CD-9902-CCD5DBAEF82F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7194859D-A7AC-4F9D-BFD7-555B51CC4CD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" firstSheet="5" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" firstSheet="3" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -215,7 +215,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="348">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="345">
   <si>
     <t>Topic</t>
   </si>
@@ -355,18 +355,84 @@
     <t>LastReviewed</t>
   </si>
   <si>
+    <t>test title</t>
+  </si>
+  <si>
+    <t>Initial example record; Jan to research and complete factual fields and source.</t>
+  </si>
+  <si>
+    <t>soraka</t>
+  </si>
+  <si>
+    <t>Soraka</t>
+  </si>
+  <si>
+    <t>Easy</t>
+  </si>
+  <si>
+    <t>Her main job is healing allies and she has simple abilities</t>
+  </si>
+  <si>
+    <t>Soraka.png</t>
+  </si>
+  <si>
+    <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/Soraka.png</t>
+  </si>
+  <si>
+    <t>leona</t>
+  </si>
+  <si>
+    <t>Leona</t>
+  </si>
+  <si>
+    <t>Easy-Medium</t>
+  </si>
+  <si>
+    <t>She is a tank support with strong crowd control and straightforward abilities</t>
+  </si>
+  <si>
+    <t>Leona.png</t>
+  </si>
+  <si>
+    <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/Leona.png</t>
+  </si>
+  <si>
+    <t>lulu</t>
+  </si>
+  <si>
+    <t>Lulu</t>
+  </si>
+  <si>
+    <t>Lulu provides shields, movment speed, and crowd control for her team</t>
+  </si>
+  <si>
+    <t>Lulu.png</t>
+  </si>
+  <si>
+    <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/Lulu.png</t>
+  </si>
+  <si>
+    <t>darius</t>
+  </si>
+  <si>
+    <t>Darius</t>
+  </si>
+  <si>
+    <t>Darius is a powerful fighter with a simple but effective kit</t>
+  </si>
+  <si>
+    <t>darius.png</t>
+  </si>
+  <si>
+    <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/Darius.png</t>
+  </si>
+  <si>
     <t>garen</t>
   </si>
   <si>
     <t>Garen</t>
   </si>
   <si>
-    <t>test title</t>
-  </si>
-  <si>
-    <t>Easy</t>
-  </si>
-  <si>
     <t>Garen has a simple abilitie kit,strong durability and no resource managment</t>
   </si>
   <si>
@@ -376,7 +442,79 @@
     <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/Garen.png</t>
   </si>
   <si>
-    <t>Initial example record; Jan to research and complete factual fields and source.</t>
+    <t>malphite</t>
+  </si>
+  <si>
+    <t>Malphite</t>
+  </si>
+  <si>
+    <t>Malphite is a tank champion with straightforward abilities and excellent survivalbility</t>
+  </si>
+  <si>
+    <t>Malphite.png</t>
+  </si>
+  <si>
+    <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/Malphite.png</t>
+  </si>
+  <si>
+    <t>warwick</t>
+  </si>
+  <si>
+    <t>Warwick</t>
+  </si>
+  <si>
+    <t>He has a strong sustain through healing, a healthy jungle clear and a passive that helps track low-health enemies</t>
+  </si>
+  <si>
+    <t>warwick.png</t>
+  </si>
+  <si>
+    <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/Warwick.png</t>
+  </si>
+  <si>
+    <t>amumu</t>
+  </si>
+  <si>
+    <t>Amumu</t>
+  </si>
+  <si>
+    <t>Amumu has simple abilities, strong crowd control, and great team fight impact</t>
+  </si>
+  <si>
+    <t>Amumu.png</t>
+  </si>
+  <si>
+    <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/Amumu.png</t>
+  </si>
+  <si>
+    <t>master-yi</t>
+  </si>
+  <si>
+    <t>Master Yi</t>
+  </si>
+  <si>
+    <t>Master Yi has a straightforward kit focused on dealing damage and farming efficiently</t>
+  </si>
+  <si>
+    <t>MasterYi.png</t>
+  </si>
+  <si>
+    <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/MasterYi.png</t>
+  </si>
+  <si>
+    <t>annie</t>
+  </si>
+  <si>
+    <t>Annie</t>
+  </si>
+  <si>
+    <t>Annie has simple abilities, reliable damage, and a powerful stun</t>
+  </si>
+  <si>
+    <t>Annie.png</t>
+  </si>
+  <si>
+    <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/Annie.png</t>
   </si>
   <si>
     <t>lux</t>
@@ -385,153 +523,6 @@
     <t>Lux</t>
   </si>
   <si>
-    <t>lux.webp</t>
-  </si>
-  <si>
-    <t>malphite</t>
-  </si>
-  <si>
-    <t>Malphite</t>
-  </si>
-  <si>
-    <t>Easy-Medium</t>
-  </si>
-  <si>
-    <t>Malphite is a tank champion with straightforward abilities and excellent survivalbility</t>
-  </si>
-  <si>
-    <t>malphite.webp</t>
-  </si>
-  <si>
-    <t>https://ddragon.leagueoflegends.com/15.18.1/img/Malphte.png</t>
-  </si>
-  <si>
-    <t>soraka</t>
-  </si>
-  <si>
-    <t>Soraka</t>
-  </si>
-  <si>
-    <t>Her main job is healing allies and she has simple abilities</t>
-  </si>
-  <si>
-    <t>Soraka.png</t>
-  </si>
-  <si>
-    <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/Soraka.png</t>
-  </si>
-  <si>
-    <t>leona</t>
-  </si>
-  <si>
-    <t>Leona</t>
-  </si>
-  <si>
-    <t>She is a tank support with strong crowd control and straightforward abilities</t>
-  </si>
-  <si>
-    <t>Leona.png</t>
-  </si>
-  <si>
-    <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/Leona.png</t>
-  </si>
-  <si>
-    <t>lulu</t>
-  </si>
-  <si>
-    <t>Lulu</t>
-  </si>
-  <si>
-    <t>Lulu provides shields, movment speed, and crowd control for her team</t>
-  </si>
-  <si>
-    <t>Lulu.png</t>
-  </si>
-  <si>
-    <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/Lulu.png</t>
-  </si>
-  <si>
-    <t>darius</t>
-  </si>
-  <si>
-    <t>Darius</t>
-  </si>
-  <si>
-    <t>Darius is a powerful fighter with a simple but effective kit</t>
-  </si>
-  <si>
-    <t>darius.png</t>
-  </si>
-  <si>
-    <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/Darius.png</t>
-  </si>
-  <si>
-    <t>Malphite.png</t>
-  </si>
-  <si>
-    <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/Malphite.png</t>
-  </si>
-  <si>
-    <t>warwick</t>
-  </si>
-  <si>
-    <t>Warwick</t>
-  </si>
-  <si>
-    <t>He has a strong sustain through healing, a healthy jungle clear and a passive that helps track low-health enemies</t>
-  </si>
-  <si>
-    <t>warwick.png</t>
-  </si>
-  <si>
-    <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/Warwick.png</t>
-  </si>
-  <si>
-    <t>amumu</t>
-  </si>
-  <si>
-    <t>Amumu</t>
-  </si>
-  <si>
-    <t>Amumu has simple abilities, strong crowd control, and great team fight impact</t>
-  </si>
-  <si>
-    <t>Amumu.png</t>
-  </si>
-  <si>
-    <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/Amumu.png</t>
-  </si>
-  <si>
-    <t>master-yi</t>
-  </si>
-  <si>
-    <t>Master Yi</t>
-  </si>
-  <si>
-    <t>Master Yi has a straightforward kit focused on dealing damage and farming efficiently</t>
-  </si>
-  <si>
-    <t>MasterYi.png</t>
-  </si>
-  <si>
-    <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/MasterYi.png</t>
-  </si>
-  <si>
-    <t>annie</t>
-  </si>
-  <si>
-    <t>Annie</t>
-  </si>
-  <si>
-    <t>Annie has simple abilities, reliable damage, and a powerful stun</t>
-  </si>
-  <si>
-    <t>Annie.png</t>
-  </si>
-  <si>
-    <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/Annie.png</t>
-  </si>
-  <si>
     <t>Lux has strong abilities,which include a stun and allow her a high damage output from a safe distance</t>
   </si>
   <si>
@@ -718,9 +709,6 @@
     <t>REC003</t>
   </si>
   <si>
-    <t>Easy-Meduim</t>
-  </si>
-  <si>
     <t>Tank</t>
   </si>
   <si>
@@ -737,6 +725,9 @@
   </si>
   <si>
     <t>conqueror</t>
+  </si>
+  <si>
+    <t>Just a test</t>
   </si>
   <si>
     <t>REC005</t>
@@ -1407,13 +1398,13 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2098,417 +2089,385 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="30.75">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>53</v>
-      </c>
       <c r="I2" s="4"/>
     </row>
     <row r="3" spans="1:9" ht="30.75">
-      <c r="A3" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>55</v>
-      </c>
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
       <c r="C3" s="3"/>
-      <c r="D3" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>56</v>
-      </c>
+      <c r="D3" s="3"/>
+      <c r="F3" s="2"/>
       <c r="H3" s="3" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="I3" s="4"/>
     </row>
     <row r="4" spans="1:9" ht="30.75">
-      <c r="A4" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>58</v>
-      </c>
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
       <c r="C4" s="3"/>
-      <c r="D4" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>62</v>
-      </c>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="5"/>
       <c r="H4" s="3" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="I4" s="4"/>
     </row>
     <row r="5" spans="1:9" ht="30.75">
       <c r="A5" s="3" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>67</v>
+        <v>53</v>
       </c>
       <c r="H5" s="3"/>
       <c r="I5" s="4"/>
     </row>
     <row r="6" spans="1:9" ht="30.75">
       <c r="A6" s="3" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>69</v>
+        <v>55</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="G6" s="5" t="s">
         <v>59</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>72</v>
       </c>
       <c r="H6" s="3"/>
       <c r="I6" s="4"/>
     </row>
     <row r="7" spans="1:9" ht="30.75">
       <c r="A7" s="3" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>74</v>
+        <v>61</v>
       </c>
       <c r="C7" s="3"/>
       <c r="D7" s="3" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>76</v>
+        <v>63</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="H7" s="3"/>
       <c r="I7" s="4"/>
     </row>
     <row r="8" spans="1:9" ht="30.75">
       <c r="A8" s="3" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="C8" s="3"/>
       <c r="D8" s="3" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>81</v>
+        <v>68</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>82</v>
+        <v>69</v>
       </c>
       <c r="H8" s="3"/>
       <c r="I8" s="4"/>
     </row>
     <row r="9" spans="1:9" ht="30.75">
       <c r="A9" s="3" t="s">
-        <v>46</v>
+        <v>70</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>47</v>
+        <v>71</v>
       </c>
       <c r="C9" s="3"/>
       <c r="D9" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>50</v>
+        <v>72</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>51</v>
+        <v>73</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>52</v>
+        <v>74</v>
       </c>
       <c r="H9" s="3"/>
       <c r="I9" s="4"/>
     </row>
     <row r="10" spans="1:9" ht="30.75">
       <c r="A10" s="3" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="C10" s="3"/>
       <c r="D10" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>60</v>
+        <v>77</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="H10" s="3"/>
       <c r="I10" s="4"/>
     </row>
     <row r="11" spans="1:9" ht="30.75">
       <c r="A11" s="3" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="H11" s="3"/>
       <c r="I11" s="4"/>
     </row>
     <row r="12" spans="1:9" ht="30.75">
       <c r="A12" s="3" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="C12" s="3"/>
       <c r="D12" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="H12" s="3"/>
       <c r="I12" s="4"/>
     </row>
     <row r="13" spans="1:9" ht="30.75">
       <c r="A13" s="3" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="C13" s="3"/>
       <c r="D13" s="3" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="H13" s="3"/>
       <c r="I13" s="4"/>
     </row>
     <row r="14" spans="1:9" ht="30.75">
       <c r="A14" s="3" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="C14" s="3"/>
       <c r="D14" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="H14" s="3"/>
       <c r="I14" s="4"/>
     </row>
     <row r="15" spans="1:9" ht="30.75">
       <c r="A15" s="3" t="s">
-        <v>54</v>
+        <v>100</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>55</v>
+        <v>101</v>
       </c>
       <c r="C15" s="3"/>
       <c r="D15" s="3" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="H15" s="3"/>
       <c r="I15" s="4"/>
     </row>
     <row r="16" spans="1:9" ht="45.75">
       <c r="A16" s="3" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C16" s="3"/>
       <c r="D16" s="3" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="H16" s="3"/>
       <c r="I16" s="4"/>
     </row>
     <row r="17" spans="1:9" ht="30.75">
       <c r="A17" s="3" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C17" s="3"/>
       <c r="D17" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H17" s="3"/>
       <c r="I17" s="4"/>
     </row>
     <row r="18" spans="1:9" ht="45.75">
       <c r="A18" s="3" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C18" s="3"/>
       <c r="D18" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="H18" s="3"/>
       <c r="I18" s="4"/>
     </row>
     <row r="19" spans="1:9" ht="30.75">
       <c r="A19" s="3" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C19" s="3"/>
       <c r="D19" s="3" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="H19" s="3"/>
       <c r="I19" s="4"/>
@@ -2522,21 +2481,19 @@
     <hyperlink ref="G12" r:id="rId5" xr:uid="{B8BEF309-A3A2-46E1-95AF-7D18A3AEE31C}"/>
     <hyperlink ref="G13" r:id="rId6" xr:uid="{AA8B2E10-1788-41CB-B862-F3FCB95F51D9}"/>
     <hyperlink ref="G8" r:id="rId7" xr:uid="{1EB11F8C-1845-4368-BE3A-6397F34E89DC}"/>
-    <hyperlink ref="G2" r:id="rId8" xr:uid="{1F476FB8-2F65-4E31-8806-2934A4D4AFF6}"/>
-    <hyperlink ref="G4" r:id="rId9" xr:uid="{5E220BED-EFE0-434F-AC54-538856FA6AC1}"/>
-    <hyperlink ref="G9" r:id="rId10" xr:uid="{40DE9256-4B6C-4A28-B1B8-E46CC9DEA8C1}"/>
-    <hyperlink ref="G10" r:id="rId11" xr:uid="{66A55C05-251C-4D30-8FA2-9BA68BC9D003}"/>
-    <hyperlink ref="G14" r:id="rId12" xr:uid="{CC017235-9635-4D45-884A-5937C10F4564}"/>
-    <hyperlink ref="G15" r:id="rId13" xr:uid="{7B4A2518-A4FF-4FB6-ABC0-6710E2D4AA4C}"/>
-    <hyperlink ref="G16" r:id="rId14" xr:uid="{071C59B2-5D86-4F6A-B33C-778CE56AD474}"/>
-    <hyperlink ref="G17" r:id="rId15" xr:uid="{15FB2263-4E8B-4387-8059-41B5699DD65E}"/>
-    <hyperlink ref="G18" r:id="rId16" xr:uid="{FA6BE657-6157-4F1A-BC8D-7F0AA899B7B8}"/>
-    <hyperlink ref="G19" r:id="rId17" xr:uid="{0B2E789A-DD8A-41AA-87E4-02A3D9943F68}"/>
+    <hyperlink ref="G9" r:id="rId8" xr:uid="{40DE9256-4B6C-4A28-B1B8-E46CC9DEA8C1}"/>
+    <hyperlink ref="G10" r:id="rId9" xr:uid="{66A55C05-251C-4D30-8FA2-9BA68BC9D003}"/>
+    <hyperlink ref="G14" r:id="rId10" xr:uid="{CC017235-9635-4D45-884A-5937C10F4564}"/>
+    <hyperlink ref="G15" r:id="rId11" xr:uid="{7B4A2518-A4FF-4FB6-ABC0-6710E2D4AA4C}"/>
+    <hyperlink ref="G16" r:id="rId12" xr:uid="{071C59B2-5D86-4F6A-B33C-778CE56AD474}"/>
+    <hyperlink ref="G17" r:id="rId13" xr:uid="{15FB2263-4E8B-4387-8059-41B5699DD65E}"/>
+    <hyperlink ref="G18" r:id="rId14" xr:uid="{FA6BE657-6157-4F1A-BC8D-7F0AA899B7B8}"/>
+    <hyperlink ref="G19" r:id="rId15" xr:uid="{0B2E789A-DD8A-41AA-87E4-02A3D9943F68}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing r:id="rId18"/>
+  <legacyDrawing r:id="rId16"/>
   <tableParts count="1">
-    <tablePart r:id="rId19"/>
+    <tablePart r:id="rId17"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2562,13 +2519,13 @@
         <v>38</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>41</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>42</v>
@@ -2579,106 +2536,106 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>130</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>133</v>
       </c>
       <c r="E2" s="2">
         <v>1</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="2" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="E3" s="2">
         <v>2</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="G3" s="2"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>139</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>142</v>
       </c>
       <c r="E4" s="2">
         <v>3</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="G4" s="2"/>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="2" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="E5" s="2">
         <v>4</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="G5" s="2"/>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="2" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="E6" s="2">
         <v>5</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="G6" s="2"/>
     </row>
@@ -2721,34 +2678,34 @@
         <v>28</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>43</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>44</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>45</v>
@@ -2756,62 +2713,62 @@
     </row>
     <row r="2" spans="1:14" ht="30.75">
       <c r="A2" s="2" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>46</v>
+        <v>70</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="D2" s="3">
         <v>5</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
       <c r="L2" s="3" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="M2" s="3"/>
       <c r="N2" s="4"/>
     </row>
     <row r="3" spans="1:14">
       <c r="A3" s="3" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D3" s="3">
         <v>5</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
@@ -2822,28 +2779,28 @@
     </row>
     <row r="4" spans="1:14">
       <c r="A4" s="3" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D4" s="3">
         <v>4</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>167</v>
+        <v>56</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
@@ -2854,62 +2811,64 @@
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="3" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D5" s="3">
         <v>4</v>
       </c>
       <c r="E5" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>171</v>
-      </c>
       <c r="G5" s="3" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="I5" s="3"/>
       <c r="J5" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="K5" s="3"/>
+        <v>169</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>170</v>
+      </c>
       <c r="L5" s="3"/>
       <c r="M5" s="3"/>
       <c r="N5" s="4"/>
     </row>
     <row r="6" spans="1:14">
       <c r="A6" s="3" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="D6" s="3">
         <v>4</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>167</v>
+        <v>56</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
@@ -2920,28 +2879,28 @@
     </row>
     <row r="7" spans="1:14">
       <c r="A7" s="3" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>46</v>
+        <v>70</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="D7" s="3">
         <v>5</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F7" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="H7" s="3" t="s">
         <v>175</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>178</v>
       </c>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
@@ -2952,28 +2911,28 @@
     </row>
     <row r="8" spans="1:14">
       <c r="A8" s="3" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="D8" s="3">
         <v>5</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
@@ -2984,28 +2943,28 @@
     </row>
     <row r="9" spans="1:14">
       <c r="A9" s="3" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D9" s="3">
         <v>5</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
@@ -3016,28 +2975,28 @@
     </row>
     <row r="10" spans="1:14">
       <c r="A10" s="3" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D10" s="3">
         <v>5</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="I10" s="3"/>
       <c r="J10" s="3"/>
@@ -3048,28 +3007,28 @@
     </row>
     <row r="11" spans="1:14">
       <c r="A11" s="3" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D11" s="3">
         <v>4</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>167</v>
+        <v>56</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="I11" s="3"/>
       <c r="J11" s="3"/>
@@ -3080,28 +3039,28 @@
     </row>
     <row r="12" spans="1:14">
       <c r="A12" s="3" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D12" s="3">
         <v>5</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="I12" s="3"/>
       <c r="J12" s="3"/>
@@ -3112,28 +3071,28 @@
     </row>
     <row r="13" spans="1:14">
       <c r="A13" s="3" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>54</v>
+        <v>100</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D13" s="3">
         <v>4</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>167</v>
+        <v>56</v>
       </c>
       <c r="F13" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="H13" s="3" t="s">
         <v>189</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>192</v>
       </c>
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
@@ -3144,28 +3103,28 @@
     </row>
     <row r="14" spans="1:14">
       <c r="A14" s="3" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D14" s="3">
         <v>4</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>167</v>
+        <v>56</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="I14" s="3"/>
       <c r="J14" s="3"/>
@@ -3176,28 +3135,28 @@
     </row>
     <row r="15" spans="1:14">
       <c r="A15" s="3" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="D15" s="3">
         <v>5</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="I15" s="3"/>
       <c r="J15" s="3"/>
@@ -3208,28 +3167,28 @@
     </row>
     <row r="16" spans="1:14">
       <c r="A16" s="3" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="D16" s="3">
         <v>5</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F16" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="H16" s="3" t="s">
         <v>196</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="H16" s="3" t="s">
-        <v>199</v>
       </c>
       <c r="I16" s="3"/>
       <c r="J16" s="3"/>
@@ -3240,28 +3199,28 @@
     </row>
     <row r="17" spans="1:14">
       <c r="A17" s="3" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="D17" s="3">
         <v>4</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>167</v>
+        <v>56</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="I17" s="3"/>
       <c r="J17" s="3"/>
@@ -3272,19 +3231,19 @@
     </row>
     <row r="18" spans="1:14">
       <c r="A18" s="3" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>46</v>
+        <v>70</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
       <c r="G18" s="3" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="H18" s="3"/>
       <c r="I18" s="3"/>
@@ -3296,28 +3255,28 @@
     </row>
     <row r="19" spans="1:14" ht="30.75">
       <c r="A19" s="3" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="D19" s="3">
         <v>5</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="I19" s="3"/>
       <c r="J19" s="3"/>
@@ -3401,7 +3360,7 @@
         <v>38</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>41</v>
@@ -3421,32 +3380,32 @@
     </row>
     <row r="2" spans="1:8" ht="30.75">
       <c r="A2" s="2" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="3"/>
       <c r="E2" s="2" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="F2" s="3"/>
       <c r="G2" s="3" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="H2" s="4"/>
     </row>
     <row r="3" spans="1:8" ht="30.75">
       <c r="A3" s="3" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
@@ -3455,14 +3414,14 @@
     </row>
     <row r="4" spans="1:8" ht="30.75">
       <c r="A4" s="3" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C4" s="3"/>
       <c r="D4" s="3" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
@@ -3471,14 +3430,14 @@
     </row>
     <row r="5" spans="1:8" ht="30.75">
       <c r="A5" s="3" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
@@ -3487,14 +3446,14 @@
     </row>
     <row r="6" spans="1:8" ht="30.75">
       <c r="A6" s="3" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="3" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
@@ -3503,14 +3462,14 @@
     </row>
     <row r="7" spans="1:8" ht="30.75">
       <c r="A7" s="3" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="C7" s="3"/>
       <c r="D7" s="3" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
@@ -3519,14 +3478,14 @@
     </row>
     <row r="8" spans="1:8" ht="30.75">
       <c r="A8" s="3" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="C8" s="3"/>
       <c r="D8" s="3" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
@@ -3535,14 +3494,14 @@
     </row>
     <row r="9" spans="1:8" ht="30.75">
       <c r="A9" s="3" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="C9" s="3"/>
       <c r="D9" s="3" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
@@ -3551,14 +3510,14 @@
     </row>
     <row r="10" spans="1:8" ht="30.75">
       <c r="A10" s="3" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="C10" s="3"/>
       <c r="D10" s="3" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
@@ -3567,14 +3526,14 @@
     </row>
     <row r="11" spans="1:8" ht="30.75">
       <c r="A11" s="3" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="3" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
@@ -3583,14 +3542,14 @@
     </row>
     <row r="12" spans="1:8" ht="30.75">
       <c r="A12" s="3" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="C12" s="3"/>
       <c r="D12" s="3" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
@@ -3599,14 +3558,14 @@
     </row>
     <row r="13" spans="1:8" ht="30.75">
       <c r="A13" s="3" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="C13" s="3"/>
       <c r="D13" s="3" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
@@ -3615,14 +3574,14 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14" s="3" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="C14" s="3"/>
       <c r="D14" s="3" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
@@ -3631,14 +3590,14 @@
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="3" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="C15" s="3"/>
       <c r="D15" s="3" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
@@ -3647,14 +3606,14 @@
     </row>
     <row r="16" spans="1:8" ht="30.75">
       <c r="A16" s="3" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="C16" s="3"/>
       <c r="D16" s="3" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
@@ -3749,7 +3708,7 @@
         <v>41</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>43</v>
@@ -3763,35 +3722,35 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" s="2" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="F2" s="3"/>
       <c r="G2" s="3" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="H2" s="4"/>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="3" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
@@ -3801,13 +3760,13 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="3" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
@@ -3817,13 +3776,13 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="3" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
@@ -4018,38 +3977,38 @@
         <v>30</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D2" s="3">
         <v>1</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="3" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3">
@@ -4059,10 +4018,10 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="3" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C4" s="3"/>
       <c r="D4" s="3">
@@ -4072,10 +4031,10 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="3" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3">
@@ -4085,10 +4044,10 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="3" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="3">
@@ -4098,10 +4057,10 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="3" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="C7" s="3"/>
       <c r="D7" s="3">
@@ -4111,10 +4070,10 @@
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="3" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C8" s="3"/>
       <c r="D8" s="3">
@@ -4124,10 +4083,10 @@
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="3" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="C9" s="3"/>
       <c r="D9" s="3">
@@ -4137,10 +4096,10 @@
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="3" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="C10" s="3"/>
       <c r="D10" s="3">
@@ -4150,10 +4109,10 @@
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="3" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="3">
@@ -4163,10 +4122,10 @@
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="3" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C12" s="3"/>
       <c r="D12" s="3">
@@ -4176,10 +4135,10 @@
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="3" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="C13" s="3"/>
       <c r="D13" s="3">
@@ -4189,10 +4148,10 @@
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="3" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="C14" s="3"/>
       <c r="D14" s="3">
@@ -4202,10 +4161,10 @@
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="3" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="C15" s="3"/>
       <c r="D15" s="3">
@@ -4215,10 +4174,10 @@
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="3" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="C16" s="3"/>
       <c r="D16" s="3">
@@ -4228,10 +4187,10 @@
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="3" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="C17" s="3"/>
       <c r="D17" s="3">
@@ -4241,10 +4200,10 @@
     </row>
     <row r="18" spans="1:5" ht="30.75">
       <c r="A18" s="3" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="C18" s="3"/>
       <c r="D18" s="3">
@@ -4254,10 +4213,10 @@
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="3" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C19" s="3"/>
       <c r="D19" s="3">
@@ -4267,10 +4226,10 @@
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="3" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C20" s="3"/>
       <c r="D20" s="3">
@@ -4280,10 +4239,10 @@
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="3" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="C21" s="3"/>
       <c r="D21" s="3">
@@ -4293,10 +4252,10 @@
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="3" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D22" s="3">
         <v>6</v>
@@ -4304,10 +4263,10 @@
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="3" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="D23" s="3">
         <v>7</v>
@@ -4336,24 +4295,24 @@
         <v>40</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D2" s="2">
         <v>1</v>
@@ -4361,13 +4320,13 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="D3" s="2">
         <v>2</v>
@@ -4375,11 +4334,11 @@
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="2" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="D4" s="2">
         <v>3</v>
@@ -4389,7 +4348,7 @@
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="D5" s="2">
         <v>4</v>
@@ -4420,22 +4379,22 @@
   <sheetData>
     <row r="1" spans="1:8" ht="30.75">
       <c r="A1" s="12" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="C1" s="13" t="s">
         <v>38</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="E1" s="13" t="s">
         <v>42</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="G1" s="13" t="s">
         <v>43</v>
@@ -4446,19 +4405,19 @@
     </row>
     <row r="2" spans="1:8" ht="30.75">
       <c r="A2" s="6" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B2" s="7" t="s">
+        <v>273</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>274</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>275</v>
+      </c>
+      <c r="E2" s="7" t="s">
         <v>276</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>277</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>278</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>279</v>
       </c>
       <c r="F2" s="7">
         <v>1</v>
@@ -4468,19 +4427,19 @@
     </row>
     <row r="3" spans="1:8" ht="45.75">
       <c r="A3" s="9" t="s">
+        <v>277</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>273</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>278</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>279</v>
+      </c>
+      <c r="E3" s="10" t="s">
         <v>280</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>276</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>281</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>282</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>283</v>
       </c>
       <c r="F3" s="10">
         <v>2</v>
@@ -4490,19 +4449,19 @@
     </row>
     <row r="4" spans="1:8" ht="30.75">
       <c r="A4" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>273</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>282</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>283</v>
+      </c>
+      <c r="E4" s="7" t="s">
         <v>284</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>276</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>285</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>286</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>287</v>
       </c>
       <c r="F4" s="7">
         <v>3</v>
@@ -4512,19 +4471,19 @@
     </row>
     <row r="5" spans="1:8" ht="30.75">
       <c r="A5" s="9" t="s">
+        <v>285</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>273</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>286</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>287</v>
+      </c>
+      <c r="E5" s="10" t="s">
         <v>288</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>276</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>289</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>290</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>291</v>
       </c>
       <c r="F5" s="10">
         <v>4</v>
@@ -4534,19 +4493,19 @@
     </row>
     <row r="6" spans="1:8" ht="45.75">
       <c r="A6" s="6" t="s">
+        <v>289</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>290</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>291</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>292</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="E6" s="7" t="s">
         <v>293</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>294</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>295</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>296</v>
       </c>
       <c r="F6" s="7">
         <v>1</v>
@@ -4556,19 +4515,19 @@
     </row>
     <row r="7" spans="1:8" ht="45.75">
       <c r="A7" s="9" t="s">
+        <v>294</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>290</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>295</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>296</v>
+      </c>
+      <c r="E7" s="10" t="s">
         <v>297</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>293</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>298</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>299</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>300</v>
       </c>
       <c r="F7" s="10">
         <v>2</v>
@@ -4578,19 +4537,19 @@
     </row>
     <row r="8" spans="1:8" ht="30.75">
       <c r="A8" s="6" t="s">
+        <v>298</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>290</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>299</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>300</v>
+      </c>
+      <c r="E8" s="7" t="s">
         <v>301</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>293</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>302</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>303</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>304</v>
       </c>
       <c r="F8" s="7">
         <v>3</v>
@@ -4600,19 +4559,19 @@
     </row>
     <row r="9" spans="1:8" ht="45.75">
       <c r="A9" s="9" t="s">
+        <v>302</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>303</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>304</v>
+      </c>
+      <c r="D9" s="10" t="s">
         <v>305</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="E9" s="10" t="s">
         <v>306</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>307</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>308</v>
-      </c>
-      <c r="E9" s="10" t="s">
-        <v>309</v>
       </c>
       <c r="F9" s="10">
         <v>1</v>
@@ -4622,19 +4581,19 @@
     </row>
     <row r="10" spans="1:8" ht="30.75">
       <c r="A10" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>303</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>308</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>309</v>
+      </c>
+      <c r="E10" s="7" t="s">
         <v>310</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>306</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>311</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>312</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>313</v>
       </c>
       <c r="F10" s="7">
         <v>2</v>
@@ -4644,19 +4603,19 @@
     </row>
     <row r="11" spans="1:8" ht="45.75">
       <c r="A11" s="9" t="s">
+        <v>311</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>303</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>312</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>313</v>
+      </c>
+      <c r="E11" s="10" t="s">
         <v>314</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>306</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>315</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>316</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>317</v>
       </c>
       <c r="F11" s="10">
         <v>3</v>
@@ -4666,19 +4625,19 @@
     </row>
     <row r="12" spans="1:8" ht="30.75">
       <c r="A12" s="6" t="s">
+        <v>315</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>303</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>316</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>317</v>
+      </c>
+      <c r="E12" s="7" t="s">
         <v>318</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>306</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>319</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>320</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>321</v>
       </c>
       <c r="F12" s="7">
         <v>4</v>
@@ -4688,19 +4647,19 @@
     </row>
     <row r="13" spans="1:8" ht="30.75">
       <c r="A13" s="9" t="s">
+        <v>319</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>320</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>321</v>
+      </c>
+      <c r="D13" s="10" t="s">
         <v>322</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="E13" s="10" t="s">
         <v>323</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>324</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>325</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>326</v>
       </c>
       <c r="F13" s="10">
         <v>1</v>
@@ -4710,19 +4669,19 @@
     </row>
     <row r="14" spans="1:8" ht="45.75">
       <c r="A14" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>325</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>326</v>
+      </c>
+      <c r="E14" s="7" t="s">
         <v>327</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>323</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>328</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>329</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>330</v>
       </c>
       <c r="F14" s="7">
         <v>2</v>
@@ -4732,19 +4691,19 @@
     </row>
     <row r="15" spans="1:8" ht="30.75">
       <c r="A15" s="9" t="s">
+        <v>328</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>320</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>329</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="E15" s="10" t="s">
         <v>331</v>
-      </c>
-      <c r="B15" s="10" t="s">
-        <v>323</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>332</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>333</v>
-      </c>
-      <c r="E15" s="10" t="s">
-        <v>334</v>
       </c>
       <c r="F15" s="10">
         <v>3</v>
@@ -4754,19 +4713,19 @@
     </row>
     <row r="16" spans="1:8" ht="30.75">
       <c r="A16" s="6" t="s">
+        <v>332</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>334</v>
+      </c>
+      <c r="D16" s="7" t="s">
         <v>335</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="E16" s="7" t="s">
         <v>336</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>337</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>338</v>
-      </c>
-      <c r="E16" s="7" t="s">
-        <v>339</v>
       </c>
       <c r="F16" s="7">
         <v>1</v>
@@ -4776,19 +4735,19 @@
     </row>
     <row r="17" spans="1:8" ht="30.75">
       <c r="A17" s="9" t="s">
+        <v>337</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>333</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>338</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>339</v>
+      </c>
+      <c r="E17" s="10" t="s">
         <v>340</v>
-      </c>
-      <c r="B17" s="10" t="s">
-        <v>336</v>
-      </c>
-      <c r="C17" s="10" t="s">
-        <v>341</v>
-      </c>
-      <c r="D17" s="10" t="s">
-        <v>342</v>
-      </c>
-      <c r="E17" s="10" t="s">
-        <v>343</v>
       </c>
       <c r="F17" s="10">
         <v>2</v>
@@ -4798,19 +4757,19 @@
     </row>
     <row r="18" spans="1:8" ht="30.75">
       <c r="A18" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>342</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>343</v>
+      </c>
+      <c r="E18" s="7" t="s">
         <v>344</v>
-      </c>
-      <c r="B18" s="7" t="s">
-        <v>336</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>345</v>
-      </c>
-      <c r="D18" s="7" t="s">
-        <v>346</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>347</v>
       </c>
       <c r="F18" s="7">
         <v>3</v>

</xml_diff>

<commit_message>
What I found that was missing
</commit_message>
<xml_diff>
--- a/data/league-new-player-data-template-populated.xlsx
+++ b/data/league-new-player-data-template-populated.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7194859D-A7AC-4F9D-BFD7-555B51CC4CD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\LoL\league-new-player-guide\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D5F2452-54E2-4242-9860-562DBE7DDAD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" firstSheet="3" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -215,7 +220,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="345">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="373">
   <si>
     <t>Topic</t>
   </si>
@@ -544,9 +549,6 @@
     <t>Malzahar.png</t>
   </si>
   <si>
-    <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/Malzahar</t>
-  </si>
-  <si>
     <t>ashe</t>
   </si>
   <si>
@@ -685,12 +687,6 @@
     <t>ReviewedBy</t>
   </si>
   <si>
-    <t>REC001</t>
-  </si>
-  <si>
-    <t>Fighter / Tank</t>
-  </si>
-  <si>
     <t>Yes</t>
   </si>
   <si>
@@ -727,9 +723,6 @@
     <t>conqueror</t>
   </si>
   <si>
-    <t>Just a test</t>
-  </si>
-  <si>
     <t>REC005</t>
   </si>
   <si>
@@ -835,9 +828,6 @@
     <t>Doran's Shield</t>
   </si>
   <si>
-    <t>dorans-shield.webp</t>
-  </si>
-  <si>
     <t>Initial filename/ID example; Jan to confirm item facts and source.</t>
   </si>
   <si>
@@ -964,15 +954,6 @@
     <t>IsPrimary</t>
   </si>
   <si>
-    <t>BUILD001</t>
-  </si>
-  <si>
-    <t>Beginner Top Build</t>
-  </si>
-  <si>
-    <t>Example build record; intern to research and populate the actual build.</t>
-  </si>
-  <si>
     <t>Initial structural example only.</t>
   </si>
   <si>
@@ -1003,9 +984,6 @@
     <t>Starting</t>
   </si>
   <si>
-    <t>Jan to research and explain why this item belongs in the build.</t>
-  </si>
-  <si>
     <t>YesNo</t>
   </si>
   <si>
@@ -1117,9 +1095,6 @@
     <t>Hail of Blades</t>
   </si>
   <si>
-    <t>Provides a rapid burst of attack speed when combat begins.</t>
-  </si>
-  <si>
     <t>hail-of-blades.webp</t>
   </si>
   <si>
@@ -1250,6 +1225,120 @@
   </si>
   <si>
     <t>first-strike.webp</t>
+  </si>
+  <si>
+    <t>Provides a rapid burst of attack speed when you hit a champion three times at the start of combat</t>
+  </si>
+  <si>
+    <t>Summon Aery helps Soraka heal allies more effectively and also adds extra damage when poking enemies with abilities</t>
+  </si>
+  <si>
+    <t>Aftershock gives her bonus defenses and deals damage around her, whenever she immobilizes a target</t>
+  </si>
+  <si>
+    <t>Summon Aery increases the strength of her shields while also providing extra poke damage against enemies.</t>
+  </si>
+  <si>
+    <t>Conqueror grants stacking damage during combat and eventually provides bonus adaptive force.</t>
+  </si>
+  <si>
+    <t>Conqueror stacks quickly during longer battles and increases his overall damage output</t>
+  </si>
+  <si>
+    <t>Grasp of the Undying provides bonus damage, healing, and permanent health increases, making him even tankier throughout the game</t>
+  </si>
+  <si>
+    <t>Lethal Tempo increases attack speed during fights, allowing Warwick to apply more damage and benefit more often from his passive healing</t>
+  </si>
+  <si>
+    <t>Aftershock gives him extra durability when diving into the enemy team, helping him survive while crowd-controlling opponents</t>
+  </si>
+  <si>
+    <t>Lethal Tempo helps Master Yi attack much faster, increasing his damage significantly</t>
+  </si>
+  <si>
+    <t>Electrocute increases Annie's burst damage, helping her quickly eliminate enemies</t>
+  </si>
+  <si>
+    <t>Arcane Comet gives Lux additional long-range damage whenever she lands her abilities</t>
+  </si>
+  <si>
+    <t>Summon Aery increases Malzahar's poke damage and works well with his damage-over-time abilities</t>
+  </si>
+  <si>
+    <t>Lethal Tempo lets Ashe fire more arrows, increasing both her damage and crowd control</t>
+  </si>
+  <si>
+    <t>Press the Attack helps Miss Fortune deal more damage after landing several attacks on the same target</t>
+  </si>
+  <si>
+    <t>Fleet Footwork gives Caitlyn healing and movement speed, helping her stay safe while poking enemies</t>
+  </si>
+  <si>
+    <t>https://ddragon.leagueoflegends.com/cdn/15.18.1/img/Malzahar.png</t>
+  </si>
+  <si>
+    <t>Main</t>
+  </si>
+  <si>
+    <t>Makes laning safer against ranged champions and difficult matchups</t>
+  </si>
+  <si>
+    <t>The slow helps Garen stay in range of opponents, so he can attack the enemy before they are abeal to flee</t>
+  </si>
+  <si>
+    <t>More attack speed increases the number of spins from Garen's E ability, resulting in higher damage</t>
+  </si>
+  <si>
+    <t>Provides extra mobility and damage while making it easier to stick to targets</t>
+  </si>
+  <si>
+    <t>Makes Garen tankier and helps him engage fights more effectively</t>
+  </si>
+  <si>
+    <t>Excellent against teams with multiple magic damage champions</t>
+  </si>
+  <si>
+    <t>Improves survivability during team fights and helps Garen stay alive while diving into enemies</t>
+  </si>
+  <si>
+    <t>Improves jungle clear speed and adds damage during fights</t>
+  </si>
+  <si>
+    <t>Excellent against AD-heavy teams and marksmen</t>
+  </si>
+  <si>
+    <t>Helps Warwick stay on targets and makes it easier to land his fear and ultimate</t>
+  </si>
+  <si>
+    <t>Boosts Warwick's already powerful self-healing</t>
+  </si>
+  <si>
+    <t>Strong against champions with significant healing</t>
+  </si>
+  <si>
+    <t>Keeps Warwick alive when diving into team fights</t>
+  </si>
+  <si>
+    <t>Allows aggressive engages without immediately losing team fight impact</t>
+  </si>
+  <si>
+    <t>Provides stronger early-game trading power and additional sustain through basic attacks</t>
+  </si>
+  <si>
+    <t>Excellent for dueling and synergizes perfectly with Warwick's sustained combat style</t>
+  </si>
+  <si>
+    <t>Strong against AD-heavy teams and many top lane opponents</t>
+  </si>
+  <si>
+    <t>Amplifies all of Warwick's healing effects</t>
+  </si>
+  <si>
+    <t>Useful against champions with significant healing</t>
+  </si>
+  <si>
+    <t>Helps Warwick engage and stick to enemy champions</t>
   </si>
 </sst>
 </file>
@@ -1259,7 +1348,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd\-mmm\-yyyy"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1295,6 +1384,12 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -1372,7 +1467,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1415,6 +1510,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1880,13 +1978,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B19"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="105" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="24" customHeight="1">
+    <row r="1" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1894,7 +1992,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
@@ -1902,7 +2000,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
@@ -1910,7 +2008,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -1918,7 +2016,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
@@ -1926,7 +2024,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
@@ -1934,7 +2032,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>12</v>
       </c>
@@ -1942,7 +2040,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>14</v>
       </c>
@@ -1950,7 +2048,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>16</v>
       </c>
@@ -1958,7 +2056,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>18</v>
       </c>
@@ -1966,7 +2064,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>20</v>
       </c>
@@ -1974,7 +2072,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>22</v>
       </c>
@@ -1982,7 +2080,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>24</v>
       </c>
@@ -1990,7 +2088,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>26</v>
       </c>
@@ -1998,7 +2096,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>28</v>
       </c>
@@ -2006,7 +2104,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>30</v>
       </c>
@@ -2014,7 +2112,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>32</v>
       </c>
@@ -2022,7 +2120,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>34</v>
       </c>
@@ -2030,7 +2128,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>36</v>
       </c>
@@ -2046,7 +2144,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:I19"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -2059,7 +2157,7 @@
     <col min="9" max="9" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="24" customHeight="1">
+    <row r="1" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>26</v>
       </c>
@@ -2088,7 +2186,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="30.75">
+    <row r="2" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="3" t="s">
@@ -2103,7 +2201,7 @@
       </c>
       <c r="I2" s="4"/>
     </row>
-    <row r="3" spans="1:9" ht="30.75">
+    <row r="3" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="3"/>
@@ -2114,7 +2212,7 @@
       </c>
       <c r="I3" s="4"/>
     </row>
-    <row r="4" spans="1:9" ht="30.75">
+    <row r="4" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="3"/>
@@ -2127,7 +2225,7 @@
       </c>
       <c r="I4" s="4"/>
     </row>
-    <row r="5" spans="1:9" ht="30.75">
+    <row r="5" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>48</v>
       </c>
@@ -2150,7 +2248,7 @@
       <c r="H5" s="3"/>
       <c r="I5" s="4"/>
     </row>
-    <row r="6" spans="1:9" ht="30.75">
+    <row r="6" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>54</v>
       </c>
@@ -2173,7 +2271,7 @@
       <c r="H6" s="3"/>
       <c r="I6" s="4"/>
     </row>
-    <row r="7" spans="1:9" ht="30.75">
+    <row r="7" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>60</v>
       </c>
@@ -2196,7 +2294,7 @@
       <c r="H7" s="3"/>
       <c r="I7" s="4"/>
     </row>
-    <row r="8" spans="1:9" ht="30.75">
+    <row r="8" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>65</v>
       </c>
@@ -2219,7 +2317,7 @@
       <c r="H8" s="3"/>
       <c r="I8" s="4"/>
     </row>
-    <row r="9" spans="1:9" ht="30.75">
+    <row r="9" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>70</v>
       </c>
@@ -2242,7 +2340,7 @@
       <c r="H9" s="3"/>
       <c r="I9" s="4"/>
     </row>
-    <row r="10" spans="1:9" ht="30.75">
+    <row r="10" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>75</v>
       </c>
@@ -2265,7 +2363,7 @@
       <c r="H10" s="3"/>
       <c r="I10" s="4"/>
     </row>
-    <row r="11" spans="1:9" ht="30.75">
+    <row r="11" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>80</v>
       </c>
@@ -2288,7 +2386,7 @@
       <c r="H11" s="3"/>
       <c r="I11" s="4"/>
     </row>
-    <row r="12" spans="1:9" ht="30.75">
+    <row r="12" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>85</v>
       </c>
@@ -2311,7 +2409,7 @@
       <c r="H12" s="3"/>
       <c r="I12" s="4"/>
     </row>
-    <row r="13" spans="1:9" ht="30.75">
+    <row r="13" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>90</v>
       </c>
@@ -2334,7 +2432,7 @@
       <c r="H13" s="3"/>
       <c r="I13" s="4"/>
     </row>
-    <row r="14" spans="1:9" ht="30.75">
+    <row r="14" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>95</v>
       </c>
@@ -2357,7 +2455,7 @@
       <c r="H14" s="3"/>
       <c r="I14" s="4"/>
     </row>
-    <row r="15" spans="1:9" ht="30.75">
+    <row r="15" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>100</v>
       </c>
@@ -2380,7 +2478,7 @@
       <c r="H15" s="3"/>
       <c r="I15" s="4"/>
     </row>
-    <row r="16" spans="1:9" ht="45.75">
+    <row r="16" spans="1:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>105</v>
       </c>
@@ -2398,76 +2496,76 @@
         <v>108</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>109</v>
+        <v>351</v>
       </c>
       <c r="H16" s="3"/>
       <c r="I16" s="4"/>
     </row>
-    <row r="17" spans="1:9" ht="30.75">
+    <row r="17" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>110</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>111</v>
       </c>
       <c r="C17" s="3"/>
       <c r="D17" s="3" t="s">
         <v>50</v>
       </c>
       <c r="E17" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="F17" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="F17" s="3" t="s">
+      <c r="G17" s="5" t="s">
         <v>113</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>114</v>
       </c>
       <c r="H17" s="3"/>
       <c r="I17" s="4"/>
     </row>
-    <row r="18" spans="1:9" ht="45.75">
+    <row r="18" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="B18" s="3" t="s">
         <v>115</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>116</v>
       </c>
       <c r="C18" s="3"/>
       <c r="D18" s="3" t="s">
         <v>50</v>
       </c>
       <c r="E18" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="F18" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="F18" s="3" t="s">
+      <c r="G18" s="5" t="s">
         <v>118</v>
-      </c>
-      <c r="G18" s="5" t="s">
-        <v>119</v>
       </c>
       <c r="H18" s="3"/>
       <c r="I18" s="4"/>
     </row>
-    <row r="19" spans="1:9" ht="30.75">
+    <row r="19" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>120</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>121</v>
       </c>
       <c r="C19" s="3"/>
       <c r="D19" s="3" t="s">
         <v>56</v>
       </c>
       <c r="E19" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="F19" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="F19" s="3" t="s">
+      <c r="G19" s="5" t="s">
         <v>123</v>
-      </c>
-      <c r="G19" s="5" t="s">
-        <v>124</v>
       </c>
       <c r="H19" s="3"/>
       <c r="I19" s="4"/>
@@ -2501,7 +2599,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
@@ -2511,7 +2609,7 @@
     <col min="7" max="7" width="42" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="24" customHeight="1">
+    <row r="1" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
@@ -2519,13 +2617,13 @@
         <v>38</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>41</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>42</v>
@@ -2534,108 +2632,108 @@
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>129</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>130</v>
       </c>
       <c r="E2" s="2">
         <v>1</v>
       </c>
       <c r="F2" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="G2" s="2"/>
+    </row>
+    <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="G2" s="2"/>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" s="2" t="s">
+      <c r="B3" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>133</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>134</v>
       </c>
       <c r="E3" s="2">
         <v>2</v>
       </c>
       <c r="F3" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="G3" s="2"/>
+    </row>
+    <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="G3" s="2"/>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" s="2" t="s">
+      <c r="B4" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>138</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>139</v>
       </c>
       <c r="E4" s="2">
         <v>3</v>
       </c>
       <c r="F4" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="G4" s="2"/>
+    </row>
+    <row r="5" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="G4" s="2"/>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" s="2" t="s">
+      <c r="B5" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>142</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>143</v>
       </c>
       <c r="E5" s="2">
         <v>4</v>
       </c>
       <c r="F5" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="G5" s="2"/>
+    </row>
+    <row r="6" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="G5" s="2"/>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" s="2" t="s">
+      <c r="B6" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>146</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>147</v>
       </c>
       <c r="E6" s="2">
         <v>5</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="G6" s="2"/>
     </row>
@@ -2651,7 +2749,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:N21"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -2667,7 +2765,7 @@
     <col min="14" max="14" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="24" customHeight="1">
+    <row r="1" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>32</v>
       </c>
@@ -2678,82 +2776,66 @@
         <v>28</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>40</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>151</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>152</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>43</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>154</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>44</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="30.75">
-      <c r="A2" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="D2" s="3">
-        <v>5</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="F2" s="3" t="s">
+    <row r="2" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="15"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="15" t="s">
         <v>157</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3" t="s">
-        <v>160</v>
       </c>
       <c r="M2" s="3"/>
       <c r="N2" s="4"/>
     </row>
-    <row r="3" spans="1:14">
+    <row r="3" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>48</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D3" s="3">
         <v>5</v>
@@ -2762,30 +2844,34 @@
         <v>50</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
+      <c r="J3" s="15" t="s">
+        <v>292</v>
+      </c>
+      <c r="K3" s="15" t="s">
+        <v>336</v>
+      </c>
       <c r="L3" s="3"/>
       <c r="M3" s="3"/>
       <c r="N3" s="4"/>
     </row>
-    <row r="4" spans="1:14">
+    <row r="4" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>54</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D4" s="3">
         <v>4</v>
@@ -2794,30 +2880,34 @@
         <v>56</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
+      <c r="J4" s="15" t="s">
+        <v>309</v>
+      </c>
+      <c r="K4" s="15" t="s">
+        <v>337</v>
+      </c>
       <c r="L4" s="3"/>
       <c r="M4" s="3"/>
       <c r="N4" s="4"/>
     </row>
-    <row r="5" spans="1:14">
+    <row r="5" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>60</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D5" s="3">
         <v>4</v>
@@ -2826,34 +2916,34 @@
         <v>56</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="I5" s="3"/>
-      <c r="J5" s="3" t="s">
-        <v>169</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>170</v>
+      <c r="J5" s="15" t="s">
+        <v>292</v>
+      </c>
+      <c r="K5" s="15" t="s">
+        <v>338</v>
       </c>
       <c r="L5" s="3"/>
       <c r="M5" s="3"/>
       <c r="N5" s="4"/>
     </row>
-    <row r="6" spans="1:14">
+    <row r="6" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>65</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D6" s="3">
         <v>4</v>
@@ -2862,30 +2952,34 @@
         <v>56</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
+      <c r="J6" s="15" t="s">
+        <v>166</v>
+      </c>
+      <c r="K6" s="15" t="s">
+        <v>339</v>
+      </c>
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
       <c r="N6" s="4"/>
     </row>
-    <row r="7" spans="1:14">
+    <row r="7" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>70</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D7" s="3">
         <v>5</v>
@@ -2894,30 +2988,34 @@
         <v>50</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>175</v>
+        <v>155</v>
+      </c>
+      <c r="H7" s="15" t="s">
+        <v>171</v>
       </c>
       <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
+      <c r="J7" s="15" t="s">
+        <v>166</v>
+      </c>
+      <c r="K7" s="15" t="s">
+        <v>340</v>
+      </c>
       <c r="L7" s="3"/>
       <c r="M7" s="3"/>
       <c r="N7" s="4"/>
     </row>
-    <row r="8" spans="1:14">
+    <row r="8" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>75</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D8" s="3">
         <v>5</v>
@@ -2926,30 +3024,34 @@
         <v>50</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
+      <c r="J8" s="15" t="s">
+        <v>314</v>
+      </c>
+      <c r="K8" s="15" t="s">
+        <v>341</v>
+      </c>
       <c r="L8" s="3"/>
       <c r="M8" s="3"/>
       <c r="N8" s="4"/>
     </row>
-    <row r="9" spans="1:14">
+    <row r="9" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>80</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D9" s="3">
         <v>5</v>
@@ -2958,30 +3060,34 @@
         <v>50</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
+      <c r="J9" s="15" t="s">
+        <v>268</v>
+      </c>
+      <c r="K9" s="15" t="s">
+        <v>342</v>
+      </c>
       <c r="L9" s="3"/>
       <c r="M9" s="3"/>
       <c r="N9" s="4"/>
     </row>
-    <row r="10" spans="1:14">
+    <row r="10" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>85</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D10" s="3">
         <v>5</v>
@@ -2990,30 +3096,34 @@
         <v>50</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
+      <c r="J10" s="15" t="s">
+        <v>309</v>
+      </c>
+      <c r="K10" s="15" t="s">
+        <v>343</v>
+      </c>
       <c r="L10" s="3"/>
       <c r="M10" s="3"/>
       <c r="N10" s="4"/>
     </row>
-    <row r="11" spans="1:14">
+    <row r="11" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>90</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D11" s="3">
         <v>4</v>
@@ -3022,30 +3132,34 @@
         <v>56</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
+      <c r="J11" s="15" t="s">
+        <v>268</v>
+      </c>
+      <c r="K11" s="15" t="s">
+        <v>344</v>
+      </c>
       <c r="L11" s="3"/>
       <c r="M11" s="3"/>
       <c r="N11" s="4"/>
     </row>
-    <row r="12" spans="1:14">
+    <row r="12" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>95</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D12" s="3">
         <v>5</v>
@@ -3054,30 +3168,34 @@
         <v>50</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="3"/>
+      <c r="J12" s="15" t="s">
+        <v>280</v>
+      </c>
+      <c r="K12" s="15" t="s">
+        <v>345</v>
+      </c>
       <c r="L12" s="3"/>
       <c r="M12" s="3"/>
       <c r="N12" s="4"/>
     </row>
-    <row r="13" spans="1:14">
+    <row r="13" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>100</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D13" s="3">
         <v>4</v>
@@ -3086,30 +3204,34 @@
         <v>56</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
+      <c r="J13" s="15" t="s">
+        <v>297</v>
+      </c>
+      <c r="K13" s="15" t="s">
+        <v>346</v>
+      </c>
       <c r="L13" s="3"/>
       <c r="M13" s="3"/>
       <c r="N13" s="4"/>
     </row>
-    <row r="14" spans="1:14">
+    <row r="14" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>105</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D14" s="3">
         <v>4</v>
@@ -3118,30 +3240,34 @@
         <v>56</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
+      <c r="J14" s="15" t="s">
+        <v>292</v>
+      </c>
+      <c r="K14" s="15" t="s">
+        <v>347</v>
+      </c>
       <c r="L14" s="3"/>
       <c r="M14" s="3"/>
       <c r="N14" s="4"/>
     </row>
-    <row r="15" spans="1:14">
+    <row r="15" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D15" s="3">
         <v>5</v>
@@ -3150,30 +3276,34 @@
         <v>50</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
+      <c r="J15" s="15" t="s">
+        <v>268</v>
+      </c>
+      <c r="K15" s="15" t="s">
+        <v>348</v>
+      </c>
       <c r="L15" s="3"/>
       <c r="M15" s="3"/>
       <c r="N15" s="4"/>
     </row>
-    <row r="16" spans="1:14">
+    <row r="16" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D16" s="3">
         <v>5</v>
@@ -3182,30 +3312,34 @@
         <v>50</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="I16" s="3"/>
-      <c r="J16" s="3"/>
-      <c r="K16" s="3"/>
+      <c r="J16" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="K16" s="15" t="s">
+        <v>349</v>
+      </c>
       <c r="L16" s="3"/>
       <c r="M16" s="3"/>
       <c r="N16" s="4"/>
     </row>
-    <row r="17" spans="1:14">
+    <row r="17" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D17" s="3">
         <v>4</v>
@@ -3214,36 +3348,40 @@
         <v>56</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="I17" s="3"/>
-      <c r="J17" s="3"/>
-      <c r="K17" s="3"/>
+      <c r="J17" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="K17" s="15" t="s">
+        <v>350</v>
+      </c>
       <c r="L17" s="3"/>
       <c r="M17" s="3"/>
       <c r="N17" s="4"/>
     </row>
-    <row r="18" spans="1:14">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>70</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
       <c r="G18" s="3" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="H18" s="3"/>
       <c r="I18" s="3"/>
@@ -3253,15 +3391,15 @@
       <c r="M18" s="3"/>
       <c r="N18" s="4"/>
     </row>
-    <row r="19" spans="1:14" ht="30.75">
+    <row r="19" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>80</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D19" s="3">
         <v>5</v>
@@ -3270,13 +3408,13 @@
         <v>50</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="I19" s="3"/>
       <c r="J19" s="3"/>
@@ -3285,7 +3423,7 @@
       <c r="M19" s="3"/>
       <c r="N19" s="4"/>
     </row>
-    <row r="20" spans="1:14">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -3301,7 +3439,7 @@
       <c r="M20" s="3"/>
       <c r="N20" s="4"/>
     </row>
-    <row r="21" spans="1:14">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
@@ -3341,7 +3479,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:H21"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="3" width="28" customWidth="1"/>
@@ -3352,7 +3490,7 @@
     <col min="8" max="8" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="24" customHeight="1">
+    <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>30</v>
       </c>
@@ -3360,7 +3498,7 @@
         <v>38</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>41</v>
@@ -3378,249 +3516,243 @@
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="30.75">
-      <c r="A2" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>205</v>
-      </c>
+    <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="3"/>
-      <c r="E2" s="2" t="s">
-        <v>206</v>
-      </c>
+      <c r="E2" s="2"/>
       <c r="F2" s="3"/>
       <c r="G2" s="3" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="H2" s="4"/>
     </row>
-    <row r="3" spans="1:8" ht="30.75">
+    <row r="3" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
       <c r="H3" s="4"/>
     </row>
-    <row r="4" spans="1:8" ht="30.75">
+    <row r="4" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="C4" s="3"/>
       <c r="D4" s="3" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
       <c r="H4" s="4"/>
     </row>
-    <row r="5" spans="1:8" ht="30.75">
+    <row r="5" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
       <c r="H5" s="4"/>
     </row>
-    <row r="6" spans="1:8" ht="30.75">
+    <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="3" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
       <c r="H6" s="4"/>
     </row>
-    <row r="7" spans="1:8" ht="30.75">
+    <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="C7" s="3"/>
       <c r="D7" s="3" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="E7" s="3"/>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
       <c r="H7" s="4"/>
     </row>
-    <row r="8" spans="1:8" ht="30.75">
+    <row r="8" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="C8" s="3"/>
       <c r="D8" s="3" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="E8" s="3"/>
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
       <c r="H8" s="4"/>
     </row>
-    <row r="9" spans="1:8" ht="30.75">
+    <row r="9" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="C9" s="3"/>
       <c r="D9" s="3" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
       <c r="H9" s="4"/>
     </row>
-    <row r="10" spans="1:8" ht="30.75">
+    <row r="10" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="C10" s="3"/>
       <c r="D10" s="3" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
       <c r="H10" s="4"/>
     </row>
-    <row r="11" spans="1:8" ht="30.75">
+    <row r="11" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="C11" s="3"/>
       <c r="D11" s="3" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
       <c r="H11" s="4"/>
     </row>
-    <row r="12" spans="1:8" ht="30.75">
+    <row r="12" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="C12" s="3"/>
       <c r="D12" s="3" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
       <c r="H12" s="4"/>
     </row>
-    <row r="13" spans="1:8" ht="30.75">
+    <row r="13" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="C13" s="3"/>
       <c r="D13" s="3" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
       <c r="H13" s="4"/>
     </row>
-    <row r="14" spans="1:8">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="C14" s="3"/>
       <c r="D14" s="3" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
       <c r="H14" s="4"/>
     </row>
-    <row r="15" spans="1:8">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="C15" s="3"/>
       <c r="D15" s="3" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
       <c r="H15" s="4"/>
     </row>
-    <row r="16" spans="1:8" ht="30.75">
+    <row r="16" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="C16" s="3"/>
       <c r="D16" s="3" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
       <c r="H16" s="4"/>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -3630,7 +3762,7 @@
       <c r="G17" s="3"/>
       <c r="H17" s="4"/>
     </row>
-    <row r="18" spans="1:8">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -3640,7 +3772,7 @@
       <c r="G18" s="3"/>
       <c r="H18" s="4"/>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -3650,7 +3782,7 @@
       <c r="G19" s="3"/>
       <c r="H19" s="4"/>
     </row>
-    <row r="20" spans="1:8">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -3660,7 +3792,7 @@
       <c r="G20" s="3"/>
       <c r="H20" s="4"/>
     </row>
-    <row r="21" spans="1:8">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
@@ -3682,7 +3814,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:H21"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
@@ -3694,7 +3826,7 @@
     <col min="8" max="8" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="24" customHeight="1">
+    <row r="1" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>34</v>
       </c>
@@ -3708,7 +3840,7 @@
         <v>41</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>43</v>
@@ -3720,37 +3852,29 @@
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
-      <c r="A2" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>250</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>251</v>
-      </c>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
       <c r="E2" s="3" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="F2" s="3"/>
       <c r="G2" s="3" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
       <c r="H2" s="4"/>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
@@ -3758,15 +3882,15 @@
       <c r="G3" s="3"/>
       <c r="H3" s="4"/>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>256</v>
+        <v>248</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
@@ -3774,15 +3898,15 @@
       <c r="G4" s="3"/>
       <c r="H4" s="4"/>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
@@ -3790,7 +3914,7 @@
       <c r="G5" s="3"/>
       <c r="H5" s="4"/>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -3800,7 +3924,7 @@
       <c r="G6" s="3"/>
       <c r="H6" s="4"/>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
@@ -3810,7 +3934,7 @@
       <c r="G7" s="3"/>
       <c r="H7" s="4"/>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -3820,7 +3944,7 @@
       <c r="G8" s="3"/>
       <c r="H8" s="4"/>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -3830,7 +3954,7 @@
       <c r="G9" s="3"/>
       <c r="H9" s="4"/>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
@@ -3840,7 +3964,7 @@
       <c r="G10" s="3"/>
       <c r="H10" s="4"/>
     </row>
-    <row r="11" spans="1:8">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -3850,7 +3974,7 @@
       <c r="G11" s="3"/>
       <c r="H11" s="4"/>
     </row>
-    <row r="12" spans="1:8">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -3860,7 +3984,7 @@
       <c r="G12" s="3"/>
       <c r="H12" s="4"/>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -3870,7 +3994,7 @@
       <c r="G13" s="3"/>
       <c r="H13" s="4"/>
     </row>
-    <row r="14" spans="1:8">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -3880,7 +4004,7 @@
       <c r="G14" s="3"/>
       <c r="H14" s="4"/>
     </row>
-    <row r="15" spans="1:8">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -3890,7 +4014,7 @@
       <c r="G15" s="3"/>
       <c r="H15" s="4"/>
     </row>
-    <row r="16" spans="1:8">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -3900,7 +4024,7 @@
       <c r="G16" s="3"/>
       <c r="H16" s="4"/>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -3910,7 +4034,7 @@
       <c r="G17" s="3"/>
       <c r="H17" s="4"/>
     </row>
-    <row r="18" spans="1:8">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -3920,7 +4044,7 @@
       <c r="G18" s="3"/>
       <c r="H18" s="4"/>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -3930,7 +4054,7 @@
       <c r="G19" s="3"/>
       <c r="H19" s="4"/>
     </row>
-    <row r="20" spans="1:8">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -3940,7 +4064,7 @@
       <c r="G20" s="3"/>
       <c r="H20" s="4"/>
     </row>
-    <row r="21" spans="1:8">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
@@ -3962,14 +4086,14 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:E23"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="3" width="18" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="24" customHeight="1">
+    <row r="1" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>34</v>
       </c>
@@ -3977,299 +4101,377 @@
         <v>30</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>261</v>
-      </c>
-      <c r="D2" s="3">
-        <v>1</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="C3" s="15" t="s">
         <v>253</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="C3" s="3"/>
       <c r="D3" s="3">
         <v>1</v>
       </c>
-      <c r="E3" s="3"/>
-    </row>
-    <row r="4" spans="1:5">
+      <c r="E3" s="15" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>209</v>
-      </c>
-      <c r="C4" s="3"/>
+        <v>204</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>352</v>
+      </c>
       <c r="D4" s="3">
         <v>2</v>
       </c>
-      <c r="E4" s="3"/>
-    </row>
-    <row r="5" spans="1:5">
+      <c r="E4" s="15" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="C5" s="3"/>
+        <v>207</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>352</v>
+      </c>
       <c r="D5" s="3">
         <v>3</v>
       </c>
-      <c r="E5" s="3"/>
-    </row>
-    <row r="6" spans="1:5">
+      <c r="E5" s="15" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>215</v>
-      </c>
-      <c r="C6" s="3"/>
+        <v>210</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>352</v>
+      </c>
       <c r="D6" s="3">
         <v>4</v>
       </c>
-      <c r="E6" s="3"/>
-    </row>
-    <row r="7" spans="1:5">
+      <c r="E6" s="15" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="C7" s="3"/>
+        <v>213</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>260</v>
+      </c>
       <c r="D7" s="3">
         <v>5</v>
       </c>
-      <c r="E7" s="3"/>
-    </row>
-    <row r="8" spans="1:5">
+      <c r="E7" s="15" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>221</v>
-      </c>
-      <c r="C8" s="3"/>
+        <v>216</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>260</v>
+      </c>
       <c r="D8" s="3">
         <v>6</v>
       </c>
-      <c r="E8" s="3"/>
-    </row>
-    <row r="9" spans="1:5">
+      <c r="E8" s="15" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="C9" s="3"/>
+        <v>219</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>260</v>
+      </c>
       <c r="D9" s="3">
         <v>7</v>
       </c>
-      <c r="E9" s="3"/>
-    </row>
-    <row r="10" spans="1:5">
+      <c r="E9" s="15" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>227</v>
-      </c>
-      <c r="C10" s="3"/>
+        <v>222</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>253</v>
+      </c>
       <c r="D10" s="3">
         <v>1</v>
       </c>
-      <c r="E10" s="3"/>
-    </row>
-    <row r="11" spans="1:5">
+      <c r="E10" s="15" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>209</v>
-      </c>
-      <c r="C11" s="3"/>
+        <v>204</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>352</v>
+      </c>
       <c r="D11" s="3">
         <v>2</v>
       </c>
-      <c r="E11" s="3"/>
-    </row>
-    <row r="12" spans="1:5">
+      <c r="E11" s="15" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>230</v>
-      </c>
-      <c r="C12" s="3"/>
+        <v>225</v>
+      </c>
+      <c r="C12" s="15" t="s">
+        <v>352</v>
+      </c>
       <c r="D12" s="3">
         <v>3</v>
       </c>
-      <c r="E12" s="3"/>
-    </row>
-    <row r="13" spans="1:5">
+      <c r="E12" s="15" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>233</v>
-      </c>
-      <c r="C13" s="3"/>
+        <v>228</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>352</v>
+      </c>
       <c r="D13" s="3">
         <v>4</v>
       </c>
-      <c r="E13" s="3"/>
-    </row>
-    <row r="14" spans="1:5">
+      <c r="E13" s="15" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>236</v>
-      </c>
-      <c r="C14" s="3"/>
+        <v>231</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>260</v>
+      </c>
       <c r="D14" s="3">
         <v>5</v>
       </c>
-      <c r="E14" s="3"/>
-    </row>
-    <row r="15" spans="1:5">
+      <c r="E14" s="15" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="C15" s="3"/>
+        <v>219</v>
+      </c>
+      <c r="C15" s="15" t="s">
+        <v>260</v>
+      </c>
       <c r="D15" s="3">
         <v>6</v>
       </c>
-      <c r="E15" s="3"/>
-    </row>
-    <row r="16" spans="1:5">
+      <c r="E15" s="15" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="C16" s="3"/>
+        <v>234</v>
+      </c>
+      <c r="C16" s="15" t="s">
+        <v>260</v>
+      </c>
       <c r="D16" s="3">
         <v>7</v>
       </c>
-      <c r="E16" s="3"/>
-    </row>
-    <row r="17" spans="1:5">
+      <c r="E16" s="15" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>242</v>
-      </c>
-      <c r="C17" s="3"/>
+        <v>237</v>
+      </c>
+      <c r="C17" s="15" t="s">
+        <v>253</v>
+      </c>
       <c r="D17" s="3">
         <v>1</v>
       </c>
-      <c r="E17" s="3"/>
-    </row>
-    <row r="18" spans="1:5" ht="30.75">
+      <c r="E17" s="15" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>245</v>
-      </c>
-      <c r="C18" s="3"/>
+        <v>240</v>
+      </c>
+      <c r="C18" s="15" t="s">
+        <v>352</v>
+      </c>
       <c r="D18" s="3">
         <v>2</v>
       </c>
-      <c r="E18" s="3"/>
-    </row>
-    <row r="19" spans="1:5">
+      <c r="E18" s="15" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>230</v>
-      </c>
-      <c r="C19" s="3"/>
+        <v>225</v>
+      </c>
+      <c r="C19" s="15" t="s">
+        <v>352</v>
+      </c>
       <c r="D19" s="3">
         <v>3</v>
       </c>
-      <c r="E19" s="3"/>
-    </row>
-    <row r="20" spans="1:5">
+      <c r="E19" s="15" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>209</v>
-      </c>
-      <c r="C20" s="3"/>
+        <v>204</v>
+      </c>
+      <c r="C20" s="15" t="s">
+        <v>352</v>
+      </c>
       <c r="D20" s="3">
         <v>4</v>
       </c>
-      <c r="E20" s="3"/>
-    </row>
-    <row r="21" spans="1:5">
+      <c r="E20" s="15" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>233</v>
-      </c>
-      <c r="C21" s="3"/>
+        <v>228</v>
+      </c>
+      <c r="C21" s="15" t="s">
+        <v>260</v>
+      </c>
       <c r="D21" s="3">
         <v>5</v>
       </c>
-      <c r="E21" s="3"/>
-    </row>
-    <row r="22" spans="1:5">
+      <c r="E21" s="15" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>236</v>
+        <v>231</v>
+      </c>
+      <c r="C22" s="15" t="s">
+        <v>260</v>
       </c>
       <c r="D22" s="3">
         <v>6</v>
       </c>
-    </row>
-    <row r="23" spans="1:5">
+      <c r="E22" s="15" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>218</v>
+        <v>213</v>
+      </c>
+      <c r="C23" s="15" t="s">
+        <v>260</v>
       </c>
       <c r="D23" s="3">
         <v>7</v>
+      </c>
+      <c r="E23" s="15" t="s">
+        <v>372</v>
       </c>
     </row>
   </sheetData>
@@ -4283,78 +4485,78 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="4" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="24" customHeight="1">
+    <row r="1" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>40</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>264</v>
+        <v>255</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>50</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
       <c r="D2" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="D3" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>267</v>
+        <v>258</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2" t="s">
-        <v>268</v>
+        <v>259</v>
       </c>
       <c r="D4" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2" t="s">
-        <v>269</v>
+        <v>260</v>
       </c>
       <c r="D5" s="2">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
@@ -4370,31 +4572,31 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{841C4449-EA12-4163-BFFB-E074DBC33876}">
   <dimension ref="A1:H18"/>
-  <sheetFormatPr defaultColWidth="49.7109375" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="49.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="30.75">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
-        <v>270</v>
+        <v>261</v>
       </c>
       <c r="B1" s="13" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="C1" s="13" t="s">
         <v>38</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="E1" s="13" t="s">
         <v>42</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G1" s="13" t="s">
         <v>43</v>
@@ -4403,21 +4605,21 @@
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="30.75">
+    <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>274</v>
+        <v>265</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="F2" s="7">
         <v>1</v>
@@ -4425,21 +4627,21 @@
       <c r="G2" s="7"/>
       <c r="H2" s="8"/>
     </row>
-    <row r="3" spans="1:8" ht="45.75">
+    <row r="3" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
-        <v>277</v>
+        <v>268</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>278</v>
+        <v>269</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>279</v>
+        <v>270</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>280</v>
+        <v>271</v>
       </c>
       <c r="F3" s="10">
         <v>2</v>
@@ -4447,21 +4649,21 @@
       <c r="G3" s="10"/>
       <c r="H3" s="11"/>
     </row>
-    <row r="4" spans="1:8" ht="30.75">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
-        <v>281</v>
+        <v>272</v>
       </c>
       <c r="B4" s="7" t="s">
+        <v>264</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>273</v>
       </c>
-      <c r="C4" s="7" t="s">
-        <v>282</v>
-      </c>
       <c r="D4" s="7" t="s">
-        <v>283</v>
+        <v>274</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>284</v>
+        <v>275</v>
       </c>
       <c r="F4" s="7">
         <v>3</v>
@@ -4469,21 +4671,21 @@
       <c r="G4" s="7"/>
       <c r="H4" s="8"/>
     </row>
-    <row r="5" spans="1:8" ht="30.75">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
-        <v>285</v>
+        <v>276</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>286</v>
+        <v>277</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>287</v>
+        <v>278</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>288</v>
+        <v>279</v>
       </c>
       <c r="F5" s="10">
         <v>4</v>
@@ -4491,21 +4693,21 @@
       <c r="G5" s="10"/>
       <c r="H5" s="11"/>
     </row>
-    <row r="6" spans="1:8" ht="45.75">
+    <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>290</v>
+        <v>281</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>291</v>
+        <v>282</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>293</v>
+        <v>284</v>
       </c>
       <c r="F6" s="7">
         <v>1</v>
@@ -4513,21 +4715,21 @@
       <c r="G6" s="7"/>
       <c r="H6" s="8"/>
     </row>
-    <row r="7" spans="1:8" ht="45.75">
+    <row r="7" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
-        <v>294</v>
+        <v>285</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>290</v>
+        <v>281</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>296</v>
+        <v>287</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>297</v>
+        <v>288</v>
       </c>
       <c r="F7" s="10">
         <v>2</v>
@@ -4535,21 +4737,21 @@
       <c r="G7" s="10"/>
       <c r="H7" s="11"/>
     </row>
-    <row r="8" spans="1:8" ht="30.75">
+    <row r="8" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
-        <v>298</v>
+        <v>289</v>
       </c>
       <c r="B8" s="7" t="s">
+        <v>281</v>
+      </c>
+      <c r="C8" s="7" t="s">
         <v>290</v>
       </c>
-      <c r="C8" s="7" t="s">
-        <v>299</v>
-      </c>
       <c r="D8" s="7" t="s">
-        <v>300</v>
+        <v>335</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>301</v>
+        <v>291</v>
       </c>
       <c r="F8" s="7">
         <v>3</v>
@@ -4557,21 +4759,21 @@
       <c r="G8" s="7"/>
       <c r="H8" s="8"/>
     </row>
-    <row r="9" spans="1:8" ht="45.75">
+    <row r="9" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>304</v>
+        <v>294</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>305</v>
+        <v>295</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>306</v>
+        <v>296</v>
       </c>
       <c r="F9" s="10">
         <v>1</v>
@@ -4579,21 +4781,21 @@
       <c r="G9" s="10"/>
       <c r="H9" s="11"/>
     </row>
-    <row r="10" spans="1:8" ht="30.75">
+    <row r="10" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
-        <v>307</v>
+        <v>297</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>308</v>
+        <v>298</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>309</v>
+        <v>299</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>310</v>
+        <v>300</v>
       </c>
       <c r="F10" s="7">
         <v>2</v>
@@ -4601,21 +4803,21 @@
       <c r="G10" s="7"/>
       <c r="H10" s="8"/>
     </row>
-    <row r="11" spans="1:8" ht="45.75">
+    <row r="11" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
-        <v>311</v>
+        <v>301</v>
       </c>
       <c r="B11" s="10" t="s">
+        <v>293</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>302</v>
+      </c>
+      <c r="D11" s="10" t="s">
         <v>303</v>
       </c>
-      <c r="C11" s="10" t="s">
-        <v>312</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>313</v>
-      </c>
       <c r="E11" s="10" t="s">
-        <v>314</v>
+        <v>304</v>
       </c>
       <c r="F11" s="10">
         <v>3</v>
@@ -4623,21 +4825,21 @@
       <c r="G11" s="10"/>
       <c r="H11" s="11"/>
     </row>
-    <row r="12" spans="1:8" ht="30.75">
+    <row r="12" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
-        <v>315</v>
+        <v>305</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>316</v>
+        <v>306</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>317</v>
+        <v>307</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>318</v>
+        <v>308</v>
       </c>
       <c r="F12" s="7">
         <v>4</v>
@@ -4645,21 +4847,21 @@
       <c r="G12" s="7"/>
       <c r="H12" s="8"/>
     </row>
-    <row r="13" spans="1:8" ht="30.75">
+    <row r="13" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="9" t="s">
-        <v>319</v>
+        <v>309</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>320</v>
+        <v>310</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>321</v>
+        <v>311</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>322</v>
+        <v>312</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>323</v>
+        <v>313</v>
       </c>
       <c r="F13" s="10">
         <v>1</v>
@@ -4667,21 +4869,21 @@
       <c r="G13" s="10"/>
       <c r="H13" s="11"/>
     </row>
-    <row r="14" spans="1:8" ht="45.75">
+    <row r="14" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
-        <v>324</v>
+        <v>314</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>320</v>
+        <v>310</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>325</v>
+        <v>315</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>326</v>
+        <v>316</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>327</v>
+        <v>317</v>
       </c>
       <c r="F14" s="7">
         <v>2</v>
@@ -4689,21 +4891,21 @@
       <c r="G14" s="7"/>
       <c r="H14" s="8"/>
     </row>
-    <row r="15" spans="1:8" ht="30.75">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="9" t="s">
-        <v>328</v>
+        <v>318</v>
       </c>
       <c r="B15" s="10" t="s">
+        <v>310</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>319</v>
+      </c>
+      <c r="D15" s="10" t="s">
         <v>320</v>
       </c>
-      <c r="C15" s="10" t="s">
-        <v>329</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>330</v>
-      </c>
       <c r="E15" s="10" t="s">
-        <v>331</v>
+        <v>321</v>
       </c>
       <c r="F15" s="10">
         <v>3</v>
@@ -4711,21 +4913,21 @@
       <c r="G15" s="10"/>
       <c r="H15" s="11"/>
     </row>
-    <row r="16" spans="1:8" ht="30.75">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
-        <v>332</v>
+        <v>322</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>333</v>
+        <v>323</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>334</v>
+        <v>324</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>335</v>
+        <v>325</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>336</v>
+        <v>326</v>
       </c>
       <c r="F16" s="7">
         <v>1</v>
@@ -4733,21 +4935,21 @@
       <c r="G16" s="7"/>
       <c r="H16" s="8"/>
     </row>
-    <row r="17" spans="1:8" ht="30.75">
+    <row r="17" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="9" t="s">
-        <v>337</v>
+        <v>327</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>333</v>
+        <v>323</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>338</v>
+        <v>328</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>339</v>
+        <v>329</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>340</v>
+        <v>330</v>
       </c>
       <c r="F17" s="10">
         <v>2</v>
@@ -4755,21 +4957,21 @@
       <c r="G17" s="10"/>
       <c r="H17" s="11"/>
     </row>
-    <row r="18" spans="1:8" ht="30.75">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="6" t="s">
-        <v>341</v>
+        <v>331</v>
       </c>
       <c r="B18" s="7" t="s">
+        <v>323</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>332</v>
+      </c>
+      <c r="D18" s="7" t="s">
         <v>333</v>
       </c>
-      <c r="C18" s="7" t="s">
-        <v>342</v>
-      </c>
-      <c r="D18" s="7" t="s">
-        <v>343</v>
-      </c>
       <c r="E18" s="7" t="s">
-        <v>344</v>
+        <v>334</v>
       </c>
       <c r="F18" s="7">
         <v>3</v>

</xml_diff>